<commit_message>
docs: mark Phase 2.3 Completed in roadmap (5 completed: 1.1, 1.2, 2.1, 2.2, 2.3)
</commit_message>
<xml_diff>
--- a/RevisionGrade_Roadmap_UPDATED.xlsx
+++ b/RevisionGrade_Roadmap_UPDATED.xlsx
@@ -1395,7 +1395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A81"/>
+  <dimension ref="A1:A82"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="133.88" customWidth="1" style="95" min="1" max="1"/>
@@ -1443,7 +1443,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="14.25" customHeight="1" s="96">
       <c r="A8" s="95" t="inlineStr">
         <is>
@@ -1451,7 +1450,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="14.25" customHeight="1" s="96">
       <c r="A10" s="95" t="inlineStr">
         <is>
@@ -1462,7 +1460,7 @@
     <row r="11" ht="14.25" customHeight="1" s="96">
       <c r="A11" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Completed: 4 items (1.1, 1.2, 2.1, 2.2)</t>
+          <t xml:space="preserve">  Completed: 5 items (1.1, 1.2, 2.1, 2.2, 2.3)</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1474,7 @@
     <row r="13" ht="14.25" customHeight="1" s="96">
       <c r="A13" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Next: 11 items</t>
+          <t xml:space="preserve">  Next: 10 items</t>
         </is>
       </c>
     </row>
@@ -1494,7 +1492,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="14.25" customHeight="1" s="96">
       <c r="A17" s="95" t="inlineStr">
         <is>
@@ -1530,7 +1527,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="14.25" customHeight="1" s="96">
       <c r="A23" s="95" t="inlineStr">
         <is>
@@ -1580,7 +1576,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31" ht="14.25" customHeight="1" s="96">
       <c r="A31" s="95" t="inlineStr">
         <is>
@@ -1617,274 +1612,281 @@
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1" s="96">
-      <c r="A36" s="95" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Canon Integration (Phase 0): NEXT</t>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Apply Integrity (2.3): COMPLETED &amp; VERIFIED (13/13 tests, 2026-03-19)</t>
         </is>
       </c>
     </row>
     <row r="37" ht="14.25" customHeight="1" s="96">
       <c r="A37" s="95" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Canon Integration (Phase 0): NEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="95" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Trust &amp; Quality Uplift: NEXT IN QUEUE</t>
         </is>
       </c>
     </row>
-    <row r="38"/>
-    <row r="39" ht="14.25" customHeight="1" s="96">
-      <c r="A39" s="95" t="inlineStr">
+    <row r="39" ht="14.25" customHeight="1" s="96"/>
+    <row r="40">
+      <c r="A40" s="95" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="40"/>
-    <row r="41" ht="14.25" customHeight="1" s="96">
-      <c r="A41" s="95" t="inlineStr">
-        <is>
-          <t>Three-Layer Execution Structure</t>
-        </is>
-      </c>
-    </row>
+    <row r="41" ht="14.25" customHeight="1" s="96"/>
     <row r="42" ht="14.25" customHeight="1" s="96">
       <c r="A42" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Layer 1 — Roadmap: direction + sequencing (this workbook)</t>
+          <t>Three-Layer Execution Structure</t>
         </is>
       </c>
     </row>
     <row r="43" ht="14.25" customHeight="1" s="96">
       <c r="A43" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Layer 2 — Sprint: atomic subtasks with verification (Sprint 0 sheet)</t>
+          <t xml:space="preserve">  Layer 1 — Roadmap: direction + sequencing (this workbook)</t>
         </is>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1" s="96">
       <c r="A44" s="95" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Layer 2 — Sprint: atomic subtasks with verification (Sprint 0 sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="95" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Layer 3 — Authority: canon enforcement at runtime (Phase 0 items)</t>
         </is>
       </c>
     </row>
-    <row r="45"/>
-    <row r="46" ht="14.25" customHeight="1" s="96">
-      <c r="A46" s="95" t="inlineStr">
-        <is>
-          <t>Governance Model</t>
-        </is>
-      </c>
-    </row>
+    <row r="46" ht="14.25" customHeight="1" s="96"/>
     <row r="47" ht="14.25" customHeight="1" s="96">
       <c r="A47" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Every roadmap item has: Success Criteria, Test Method, Canon Reference</t>
+          <t>Governance Model</t>
         </is>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1" s="96">
       <c r="A48" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Every sprint subtask has: Success Criteria, Test Method, Output Artifact</t>
+          <t xml:space="preserve">  Every roadmap item has: Success Criteria, Test Method, Canon Reference</t>
         </is>
       </c>
     </row>
     <row r="49" ht="14.25" customHeight="1" s="96">
       <c r="A49" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Definition of done: "This passed its defined success test" — not "I think this is done"</t>
+          <t xml:space="preserve">  Every sprint subtask has: Success Criteria, Test Method, Output Artifact</t>
         </is>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1" s="96">
       <c r="A50" s="95" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Definition of done: "This passed its defined success test" — not "I think this is done"</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="95" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Canon compliance check required before any phase can be marked verified</t>
         </is>
       </c>
     </row>
-    <row r="51"/>
-    <row r="52" ht="14.25" customHeight="1" s="96">
-      <c r="A52" s="95" t="inlineStr">
-        <is>
-          <t>Active Gates</t>
-        </is>
-      </c>
-    </row>
+    <row r="52" ht="14.25" customHeight="1" s="96"/>
     <row r="53" ht="14.25" customHeight="1" s="96">
       <c r="A53" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2.1 DB Verification: phase21-db-verification.sql must pass before 2.2 begins</t>
+          <t>Active Gates</t>
         </is>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1" s="96">
       <c r="A54" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Canon Gate (Pass 1.5): Must execute before results surface to users</t>
+          <t xml:space="preserve">  2.1 DB Verification: phase21-db-verification.sql must pass before 2.2 begins</t>
         </is>
       </c>
     </row>
     <row r="55" ht="14.25" customHeight="1" s="96">
       <c r="A55" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Two-AI Independence: Pass 2 must never receive Pass 1 outputs</t>
+          <t xml:space="preserve">  Canon Gate (Pass 1.5): Must execute before results surface to users</t>
         </is>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1" s="96">
       <c r="A56" s="95" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Two-AI Independence: Pass 2 must never receive Pass 1 outputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="95" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Audit Spine: Append-only, hash-chained, no DELETE/UPDATE, 7-year retention</t>
         </is>
       </c>
     </row>
-    <row r="57"/>
-    <row r="58" ht="14.25" customHeight="1" s="96">
-      <c r="A58" s="95" t="inlineStr">
+    <row r="58" ht="14.25" customHeight="1" s="96"/>
+    <row r="59">
+      <c r="A59" s="95" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="59"/>
-    <row r="60" ht="14.25" customHeight="1" s="96">
-      <c r="A60" s="95" t="inlineStr">
-        <is>
-          <t>Workbook Sheets</t>
-        </is>
-      </c>
-    </row>
+    <row r="60" ht="14.25" customHeight="1" s="96"/>
     <row r="61" ht="14.25" customHeight="1" s="96">
       <c r="A61" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Overview: Dashboard with KPI cards and phase progress</t>
+          <t>Workbook Sheets</t>
         </is>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1" s="96">
       <c r="A62" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Roadmap: Full 44-item sequential tracker with all PM fields + Canon Reference</t>
+          <t xml:space="preserve">  Overview: Dashboard with KPI cards and phase progress</t>
         </is>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1" s="96">
       <c r="A63" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Sprint 0 (Phase 2): 13 atomic subtasks for 2.1-2.4 with Success/Test/Artifact</t>
+          <t xml:space="preserve">  Roadmap: Full 44-item sequential tracker with all PM fields + Canon Reference</t>
         </is>
       </c>
     </row>
     <row r="64" ht="14.25" customHeight="1" s="96">
       <c r="A64" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Immediate Priorities: The 'next three' critical deliverables</t>
+          <t xml:space="preserve">  Sprint 0 (Phase 2): 13 atomic subtasks for 2.1-2.4 with Success/Test/Artifact</t>
         </is>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1" s="96">
       <c r="A65" s="95" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Immediate Priorities: The 'next three' critical deliverables</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="95" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Canon Reference: Authority chain, numeric constants, 10 non-negotiable governance rules</t>
         </is>
       </c>
     </row>
-    <row r="66"/>
-    <row r="67" ht="14.25" customHeight="1" s="96">
-      <c r="A67" s="95" t="inlineStr">
+    <row r="67" ht="14.25" customHeight="1" s="96"/>
+    <row r="68">
+      <c r="A68" s="95" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="68"/>
-    <row r="69" ht="14.25" customHeight="1" s="96">
-      <c r="A69" s="95" t="inlineStr">
-        <is>
-          <t>Canon Document Sources (20 documents integrated)</t>
-        </is>
-      </c>
-    </row>
+    <row r="69" ht="14.25" customHeight="1" s="96"/>
     <row r="70" ht="14.25" customHeight="1" s="96">
       <c r="A70" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume I — WAVE Revision Guide Canon (62 waves, 3 tsunamis, 10 execution rules)</t>
+          <t>Canon Document Sources (20 documents integrated)</t>
         </is>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1" s="96">
       <c r="A71" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume II — Story Evaluation Criteria (13 criteria, 10 diagnostic patterns)</t>
+          <t xml:space="preserve">  Volume I — WAVE Revision Guide Canon (62 waves, 3 tsunamis, 10 execution rules)</t>
         </is>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1" s="96">
       <c r="A72" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume II-A — Operational Schema (weights, gates, JSON envelope, Supabase tables)</t>
+          <t xml:space="preserve">  Volume II — Story Evaluation Criteria (13 criteria, 10 diagnostic patterns)</t>
         </is>
       </c>
     </row>
     <row r="73" ht="14.25" customHeight="1" s="96">
       <c r="A73" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume III — Platform Governance Canon (5 doctrines, 3-layer editorial intelligence)</t>
+          <t xml:space="preserve">  Volume II-A — Operational Schema (weights, gates, JSON envelope, Supabase tables)</t>
         </is>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1" s="96">
       <c r="A74" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume III — Tools &amp; Implementation Systems (schemas, prompts, adapters)</t>
+          <t xml:space="preserve">  Volume III — Platform Governance Canon (5 doctrines, 3-layer editorial intelligence)</t>
         </is>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1" s="96">
       <c r="A75" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume III — Operational Specification (thresholds, routing, 7-stage pipeline)</t>
+          <t xml:space="preserve">  Volume III — Tools &amp; Implementation Systems (schemas, prompts, adapters)</t>
         </is>
       </c>
     </row>
     <row r="76" ht="14.25" customHeight="1" s="96">
       <c r="A76" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume IV — AI Governance Canon (3-layer authority, 7 protection systems)</t>
+          <t xml:space="preserve">  Volume III — Operational Specification (thresholds, routing, 7-stage pipeline)</t>
         </is>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1" s="96">
       <c r="A77" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume V — Execution Architecture (AEP 6-step flow, Trifecta, chunking, reliability)</t>
+          <t xml:space="preserve">  Volume IV — AI Governance Canon (3-layer authority, 7 protection systems)</t>
         </is>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1" s="96">
       <c r="A78" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Canon III — Lessons of the Living System (8 governing laws)</t>
+          <t xml:space="preserve">  Volume V — Execution Architecture (AEP 6-step flow, Trifecta, chunking, reliability)</t>
         </is>
       </c>
     </row>
     <row r="79" ht="14.25" customHeight="1" s="96">
       <c r="A79" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Canon Assembly Matrix (RCAM v2.0, 24 source docs, 5 matrix rules)</t>
+          <t xml:space="preserve">  Canon III — Lessons of the Living System (8 governing laws)</t>
         </is>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1" s="96">
       <c r="A80" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Canon Doctrine Registry (77 doctrine units, 6 governance rules)</t>
+          <t xml:space="preserve">  Canon Assembly Matrix (RCAM v2.0, 24 source docs, 5 matrix rules)</t>
         </is>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1" s="96">
       <c r="A81" s="95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Canon Doctrine Registry (77 doctrine units, 6 governance rules)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="95" t="inlineStr">
         <is>
           <t xml:space="preserve">  + 9 supporting/variant documents (txt, md formats)</t>
         </is>
@@ -1904,7 +1906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="B2:J28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="95" min="1" max="1"/>
@@ -1916,7 +1918,6 @@
     <col width="15" customWidth="1" style="95" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="36" customHeight="1" s="96">
       <c r="B2" s="98" t="inlineStr">
         <is>
@@ -1938,7 +1939,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="24" customHeight="1" s="96">
       <c r="B6" s="101" t="inlineStr">
         <is>
@@ -1946,7 +1946,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="24" customHeight="1" s="96">
       <c r="B8" s="102" t="inlineStr">
         <is>
@@ -2005,8 +2004,6 @@
         <v/>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12" ht="24" customHeight="1" s="96">
       <c r="B12" s="101" t="inlineStr">
         <is>
@@ -2014,7 +2011,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="24" customHeight="1" s="96">
       <c r="B14" s="114" t="inlineStr">
         <is>
@@ -2174,7 +2170,6 @@
         <v/>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="15" customHeight="1" s="96">
       <c r="B22" s="95" t="n"/>
     </row>
@@ -2990,7 +2985,7 @@
       <c r="E9" s="137" t="n"/>
       <c r="F9" s="147" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="G9" s="139" t="inlineStr">
@@ -7008,7 +7003,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="B2:J11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="95" min="1" max="1"/>
@@ -7020,7 +7015,6 @@
     <col width="10" customWidth="1" style="95" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="30" customHeight="1" s="96">
       <c r="B2" s="175" t="inlineStr">
         <is>
@@ -7035,7 +7029,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="25.5" customHeight="1" s="96">
       <c r="B5" s="125" t="inlineStr">
         <is>
@@ -7218,8 +7211,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10"/>
     <row r="11" ht="14.25" customHeight="1" s="96">
       <c r="B11" s="123" t="inlineStr">
         <is>
@@ -7248,7 +7239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="B2:H63"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="95" min="1" max="1"/>
@@ -7258,7 +7249,6 @@
     <col width="15" customWidth="1" style="95" min="5" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="30" customHeight="1" s="96">
       <c r="B2" s="175" t="inlineStr">
         <is>
@@ -7273,7 +7263,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="96">
       <c r="B5" s="101" t="inlineStr">
         <is>
@@ -7434,8 +7423,6 @@
       <c r="G14" s="170" t="n"/>
       <c r="H14" s="170" t="n"/>
     </row>
-    <row r="15"/>
-    <row r="16"/>
     <row r="17" ht="24" customHeight="1" s="96">
       <c r="B17" s="101" t="inlineStr">
         <is>
@@ -7953,8 +7940,6 @@
         </is>
       </c>
     </row>
-    <row r="48"/>
-    <row r="49"/>
     <row r="50" ht="24" customHeight="1" s="96">
       <c r="B50" s="101" t="inlineStr">
         <is>
@@ -8132,8 +8117,6 @@
       <c r="G60" s="170" t="n"/>
       <c r="H60" s="170" t="n"/>
     </row>
-    <row r="61"/>
-    <row r="62"/>
     <row r="63" ht="15" customHeight="1" s="96">
       <c r="B63" s="123" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: mark Phase 2.4 Completed, fill Sprint 0 subtasks, update counts (6 completed: 1.1-2.4)
</commit_message>
<xml_diff>
--- a/RevisionGrade_Roadmap_UPDATED.xlsx
+++ b/RevisionGrade_Roadmap_UPDATED.xlsx
@@ -1395,7 +1395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A82"/>
+  <dimension ref="A1:A83"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="133.88" customWidth="1" style="95" min="1" max="1"/>
@@ -1460,7 +1460,7 @@
     <row r="11" ht="14.25" customHeight="1" s="96">
       <c r="A11" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Completed: 5 items (1.1, 1.2, 2.1, 2.2, 2.3)</t>
+          <t xml:space="preserve">  Completed: 6 items (1.1, 1.2, 2.1, 2.2, 2.3, 2.4)</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1474,7 @@
     <row r="13" ht="14.25" customHeight="1" s="96">
       <c r="A13" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Next: 10 items</t>
+          <t xml:space="preserve">  Next: 9 items</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1" s="96">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="95" t="inlineStr">
         <is>
           <t xml:space="preserve">  Apply Integrity (2.3): COMPLETED &amp; VERIFIED (13/13 tests, 2026-03-19)</t>
         </is>
@@ -1621,272 +1621,276 @@
     <row r="37" ht="14.25" customHeight="1" s="96">
       <c r="A37" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Canon Integration (Phase 0): NEXT</t>
+          <t xml:space="preserve">  Failure Classification + Engine Hardening (2.4): COMPLETED &amp; VERIFIED (10 suites/100 tests, Pack F 100k soak, abe6146, 2026-03-19)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="95" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Canon Integration (Phase 0): NEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="14.25" customHeight="1" s="96">
+      <c r="A39" s="95" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Trust &amp; Quality Uplift: NEXT IN QUEUE</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="14.25" customHeight="1" s="96"/>
-    <row r="40">
-      <c r="A40" s="95" t="inlineStr">
+    <row r="41" ht="14.25" customHeight="1" s="96">
+      <c r="A41" s="95" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="14.25" customHeight="1" s="96"/>
-    <row r="42" ht="14.25" customHeight="1" s="96">
-      <c r="A42" s="95" t="inlineStr">
-        <is>
-          <t>Three-Layer Execution Structure</t>
-        </is>
-      </c>
-    </row>
+    <row r="42" ht="14.25" customHeight="1" s="96"/>
     <row r="43" ht="14.25" customHeight="1" s="96">
       <c r="A43" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Layer 1 — Roadmap: direction + sequencing (this workbook)</t>
+          <t>Three-Layer Execution Structure</t>
         </is>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1" s="96">
       <c r="A44" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Layer 2 — Sprint: atomic subtasks with verification (Sprint 0 sheet)</t>
+          <t xml:space="preserve">  Layer 1 — Roadmap: direction + sequencing (this workbook)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="95" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Layer 2 — Sprint: atomic subtasks with verification (Sprint 0 sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="14.25" customHeight="1" s="96">
+      <c r="A46" s="95" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Layer 3 — Authority: canon enforcement at runtime (Phase 0 items)</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="14.25" customHeight="1" s="96"/>
-    <row r="47" ht="14.25" customHeight="1" s="96">
-      <c r="A47" s="95" t="inlineStr">
-        <is>
-          <t>Governance Model</t>
-        </is>
-      </c>
-    </row>
+    <row r="47" ht="14.25" customHeight="1" s="96"/>
     <row r="48" ht="14.25" customHeight="1" s="96">
       <c r="A48" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Every roadmap item has: Success Criteria, Test Method, Canon Reference</t>
+          <t>Governance Model</t>
         </is>
       </c>
     </row>
     <row r="49" ht="14.25" customHeight="1" s="96">
       <c r="A49" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Every sprint subtask has: Success Criteria, Test Method, Output Artifact</t>
+          <t xml:space="preserve">  Every roadmap item has: Success Criteria, Test Method, Canon Reference</t>
         </is>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1" s="96">
       <c r="A50" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Definition of done: "This passed its defined success test" — not "I think this is done"</t>
+          <t xml:space="preserve">  Every sprint subtask has: Success Criteria, Test Method, Output Artifact</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="95" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Definition of done: "This passed its defined success test" — not "I think this is done"</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="14.25" customHeight="1" s="96">
+      <c r="A52" s="95" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Canon compliance check required before any phase can be marked verified</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="14.25" customHeight="1" s="96"/>
-    <row r="53" ht="14.25" customHeight="1" s="96">
-      <c r="A53" s="95" t="inlineStr">
-        <is>
-          <t>Active Gates</t>
-        </is>
-      </c>
-    </row>
+    <row r="53" ht="14.25" customHeight="1" s="96"/>
     <row r="54" ht="14.25" customHeight="1" s="96">
       <c r="A54" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2.1 DB Verification: phase21-db-verification.sql must pass before 2.2 begins</t>
+          <t>Active Gates</t>
         </is>
       </c>
     </row>
     <row r="55" ht="14.25" customHeight="1" s="96">
       <c r="A55" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Canon Gate (Pass 1.5): Must execute before results surface to users</t>
+          <t xml:space="preserve">  2.1 DB Verification: phase21-db-verification.sql must pass before 2.2 begins</t>
         </is>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1" s="96">
       <c r="A56" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Two-AI Independence: Pass 2 must never receive Pass 1 outputs</t>
+          <t xml:space="preserve">  Canon Gate (Pass 1.5): Must execute before results surface to users</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="95" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Two-AI Independence: Pass 2 must never receive Pass 1 outputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="14.25" customHeight="1" s="96">
+      <c r="A58" s="95" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Audit Spine: Append-only, hash-chained, no DELETE/UPDATE, 7-year retention</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="14.25" customHeight="1" s="96"/>
-    <row r="59">
-      <c r="A59" s="95" t="inlineStr">
+    <row r="60" ht="14.25" customHeight="1" s="96">
+      <c r="A60" s="95" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="14.25" customHeight="1" s="96"/>
-    <row r="61" ht="14.25" customHeight="1" s="96">
-      <c r="A61" s="95" t="inlineStr">
-        <is>
-          <t>Workbook Sheets</t>
-        </is>
-      </c>
-    </row>
+    <row r="61" ht="14.25" customHeight="1" s="96"/>
     <row r="62" ht="14.25" customHeight="1" s="96">
       <c r="A62" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Overview: Dashboard with KPI cards and phase progress</t>
+          <t>Workbook Sheets</t>
         </is>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1" s="96">
       <c r="A63" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Roadmap: Full 44-item sequential tracker with all PM fields + Canon Reference</t>
+          <t xml:space="preserve">  Overview: Dashboard with KPI cards and phase progress</t>
         </is>
       </c>
     </row>
     <row r="64" ht="14.25" customHeight="1" s="96">
       <c r="A64" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Sprint 0 (Phase 2): 13 atomic subtasks for 2.1-2.4 with Success/Test/Artifact</t>
+          <t xml:space="preserve">  Roadmap: Full 44-item sequential tracker with all PM fields + Canon Reference</t>
         </is>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1" s="96">
       <c r="A65" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Immediate Priorities: The 'next three' critical deliverables</t>
+          <t xml:space="preserve">  Sprint 0 (Phase 2): 13 atomic subtasks for 2.1-2.4 with Success/Test/Artifact</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="95" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Immediate Priorities: The 'next three' critical deliverables</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="14.25" customHeight="1" s="96">
+      <c r="A67" s="95" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Canon Reference: Authority chain, numeric constants, 10 non-negotiable governance rules</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="14.25" customHeight="1" s="96"/>
-    <row r="68">
-      <c r="A68" s="95" t="inlineStr">
+    <row r="69" ht="14.25" customHeight="1" s="96">
+      <c r="A69" s="95" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="14.25" customHeight="1" s="96"/>
-    <row r="70" ht="14.25" customHeight="1" s="96">
-      <c r="A70" s="95" t="inlineStr">
-        <is>
-          <t>Canon Document Sources (20 documents integrated)</t>
-        </is>
-      </c>
-    </row>
+    <row r="70" ht="14.25" customHeight="1" s="96"/>
     <row r="71" ht="14.25" customHeight="1" s="96">
       <c r="A71" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume I — WAVE Revision Guide Canon (62 waves, 3 tsunamis, 10 execution rules)</t>
+          <t>Canon Document Sources (20 documents integrated)</t>
         </is>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1" s="96">
       <c r="A72" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume II — Story Evaluation Criteria (13 criteria, 10 diagnostic patterns)</t>
+          <t xml:space="preserve">  Volume I — WAVE Revision Guide Canon (62 waves, 3 tsunamis, 10 execution rules)</t>
         </is>
       </c>
     </row>
     <row r="73" ht="14.25" customHeight="1" s="96">
       <c r="A73" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume II-A — Operational Schema (weights, gates, JSON envelope, Supabase tables)</t>
+          <t xml:space="preserve">  Volume II — Story Evaluation Criteria (13 criteria, 10 diagnostic patterns)</t>
         </is>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1" s="96">
       <c r="A74" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume III — Platform Governance Canon (5 doctrines, 3-layer editorial intelligence)</t>
+          <t xml:space="preserve">  Volume II-A — Operational Schema (weights, gates, JSON envelope, Supabase tables)</t>
         </is>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1" s="96">
       <c r="A75" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume III — Tools &amp; Implementation Systems (schemas, prompts, adapters)</t>
+          <t xml:space="preserve">  Volume III — Platform Governance Canon (5 doctrines, 3-layer editorial intelligence)</t>
         </is>
       </c>
     </row>
     <row r="76" ht="14.25" customHeight="1" s="96">
       <c r="A76" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume III — Operational Specification (thresholds, routing, 7-stage pipeline)</t>
+          <t xml:space="preserve">  Volume III — Tools &amp; Implementation Systems (schemas, prompts, adapters)</t>
         </is>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1" s="96">
       <c r="A77" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume IV — AI Governance Canon (3-layer authority, 7 protection systems)</t>
+          <t xml:space="preserve">  Volume III — Operational Specification (thresholds, routing, 7-stage pipeline)</t>
         </is>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1" s="96">
       <c r="A78" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume V — Execution Architecture (AEP 6-step flow, Trifecta, chunking, reliability)</t>
+          <t xml:space="preserve">  Volume IV — AI Governance Canon (3-layer authority, 7 protection systems)</t>
         </is>
       </c>
     </row>
     <row r="79" ht="14.25" customHeight="1" s="96">
       <c r="A79" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Canon III — Lessons of the Living System (8 governing laws)</t>
+          <t xml:space="preserve">  Volume V — Execution Architecture (AEP 6-step flow, Trifecta, chunking, reliability)</t>
         </is>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1" s="96">
       <c r="A80" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Canon Assembly Matrix (RCAM v2.0, 24 source docs, 5 matrix rules)</t>
+          <t xml:space="preserve">  Canon III — Lessons of the Living System (8 governing laws)</t>
         </is>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1" s="96">
       <c r="A81" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Canon Doctrine Registry (77 doctrine units, 6 governance rules)</t>
+          <t xml:space="preserve">  Canon Assembly Matrix (RCAM v2.0, 24 source docs, 5 matrix rules)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Canon Doctrine Registry (77 doctrine units, 6 governance rules)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="95" t="inlineStr">
         <is>
           <t xml:space="preserve">  + 9 supporting/variant documents (txt, md formats)</t>
         </is>
@@ -3069,7 +3073,7 @@
       <c r="E10" s="143" t="n"/>
       <c r="F10" s="147" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="G10" s="144" t="inlineStr">
@@ -3124,7 +3128,7 @@
       </c>
       <c r="Q10" s="145" t="inlineStr">
         <is>
-          <t>Feeds directly into 2.3 refinement loop. When apply fails, this is how you diagnose and fix. Output Artifacts: error enum (lib/errors/failureCodes.ts), failure migration, failure test logs.</t>
+          <t>COMPLETED at abe6146. Engine hardening: 10 suites/100 tests. Pack A (27 tests), Pack C (24 tests), Pack D (182/182 valid, 0 wrong-location), Pack F (100k soak: 0 unclassified, 0 wrong-location, 0 lost writes). Fail-closed malformed-candidate fix shipped. Operations docs spine published.</t>
         </is>
       </c>
       <c r="R10" s="141" t="inlineStr">
@@ -5913,7 +5917,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47" ht="15" customHeight="1" s="96">
       <c r="A47" s="123" t="inlineStr">
         <is>
@@ -6706,15 +6709,51 @@
           <t>S0-Apply-Engine</t>
         </is>
       </c>
-      <c r="B17" s="170" t="n"/>
-      <c r="C17" s="170" t="n"/>
-      <c r="D17" s="170" t="n"/>
-      <c r="E17" s="170" t="n"/>
-      <c r="F17" s="170" t="n"/>
-      <c r="G17" s="170" t="n"/>
-      <c r="H17" s="170" t="n"/>
-      <c r="I17" s="170" t="n"/>
-      <c r="J17" s="171" t="n"/>
+      <c r="B17" s="95" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="C17" s="95" t="inlineStr">
+        <is>
+          <t>Failure Classification</t>
+        </is>
+      </c>
+      <c r="D17" s="95" t="inlineStr">
+        <is>
+          <t>2.4.a</t>
+        </is>
+      </c>
+      <c r="E17" s="95" t="inlineStr">
+        <is>
+          <t>Enumerate failure codes</t>
+        </is>
+      </c>
+      <c r="F17" s="95" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G17" s="95" t="inlineStr">
+        <is>
+          <t>docs/errors/, lib/errors/failureCodes.ts</t>
+        </is>
+      </c>
+      <c r="H17" s="95" t="inlineStr">
+        <is>
+          <t>Closed set of failure codes (ANCHOR_MISS, CONFLICT, PARSE_ERROR, INVARIANT_VIOLATION). No UNKNOWN or empty types.</t>
+        </is>
+      </c>
+      <c r="I17" s="95" t="inlineStr">
+        <is>
+          <t>Review code for any untyped throw/catch. Grep for unknown failure strings.</t>
+        </is>
+      </c>
+      <c r="J17" s="95" t="inlineStr">
+        <is>
+          <t>lib/errors/failureCodes.ts, PACK_F_EXECUTION_CONTRACT.md</t>
+        </is>
+      </c>
       <c r="K17" s="168" t="n"/>
       <c r="L17" s="168" t="n"/>
       <c r="M17" s="168" t="n"/>
@@ -6732,17 +6771,51 @@
           <t>S0-Apply-Engine</t>
         </is>
       </c>
-      <c r="B18" s="142" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="C18" s="170" t="n"/>
-      <c r="D18" s="170" t="n"/>
-      <c r="E18" s="170" t="n"/>
-      <c r="F18" s="170" t="n"/>
-      <c r="G18" s="170" t="n"/>
-      <c r="H18" s="170" t="n"/>
-      <c r="I18" s="170" t="n"/>
-      <c r="J18" s="171" t="n"/>
+      <c r="B18" s="142" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="C18" s="95" t="inlineStr">
+        <is>
+          <t>Failure Classification</t>
+        </is>
+      </c>
+      <c r="D18" s="95" t="inlineStr">
+        <is>
+          <t>2.4.b</t>
+        </is>
+      </c>
+      <c r="E18" s="95" t="inlineStr">
+        <is>
+          <t>Wire codes into revision_sessions + telemetry</t>
+        </is>
+      </c>
+      <c r="F18" s="95" t="inlineStr">
+        <is>
+          <t>Backend / DB</t>
+        </is>
+      </c>
+      <c r="G18" s="95" t="inlineStr">
+        <is>
+          <t>supabase/migrations, lib/db/revisionSessions.ts, lib/revision/telemetry.ts</t>
+        </is>
+      </c>
+      <c r="H18" s="95" t="inlineStr">
+        <is>
+          <t>Every failed apply stores a specific failure code + context. Telemetry event codes cover all apply paths.</t>
+        </is>
+      </c>
+      <c r="I18" s="95" t="inlineStr">
+        <is>
+          <t>Run all apply paths (valid, invalid offsets, overlap, stale anchor). Verify DB row has non-null failure_code.</t>
+        </is>
+      </c>
+      <c r="J18" s="95" t="inlineStr">
+        <is>
+          <t>Updated revision_sessions schema, telemetry.ts event codes</t>
+        </is>
+      </c>
       <c r="K18" s="168" t="n"/>
       <c r="L18" s="168" t="n"/>
       <c r="M18" s="168" t="n"/>
@@ -6760,17 +6833,51 @@
           <t>S0-Apply-Engine</t>
         </is>
       </c>
-      <c r="B19" s="136" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="C19" s="170" t="n"/>
-      <c r="D19" s="170" t="n"/>
-      <c r="E19" s="170" t="n"/>
-      <c r="F19" s="170" t="n"/>
-      <c r="G19" s="170" t="n"/>
-      <c r="H19" s="170" t="n"/>
-      <c r="I19" s="170" t="n"/>
-      <c r="J19" s="171" t="n"/>
+      <c r="B19" s="136" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="C19" s="95" t="inlineStr">
+        <is>
+          <t>Failure Classification</t>
+        </is>
+      </c>
+      <c r="D19" s="95" t="inlineStr">
+        <is>
+          <t>2.4.c</t>
+        </is>
+      </c>
+      <c r="E19" s="95" t="inlineStr">
+        <is>
+          <t>Tests: 100% classified failures + Pack F soak qualification</t>
+        </is>
+      </c>
+      <c r="F19" s="95" t="inlineStr">
+        <is>
+          <t>Tests / Harness</t>
+        </is>
+      </c>
+      <c r="G19" s="95" t="inlineStr">
+        <is>
+          <t>tests/failures/, tests/operations/, scripts/soak/</t>
+        </is>
+      </c>
+      <c r="H19" s="95" t="inlineStr">
+        <is>
+          <t>10 suites/100 tests green. Pack F 100k soak: 0 unclassified, 0 wrong-location, 0 lost writes.</t>
+        </is>
+      </c>
+      <c r="I19" s="95" t="inlineStr">
+        <is>
+          <t>npm test (full suite). npm run soak:run with 1k/10k/100k events. Verify archived evidence ladder.</t>
+        </is>
+      </c>
+      <c r="J19" s="95" t="inlineStr">
+        <is>
+          <t>soak-harness.test.ts, packF archives (1k/10k/100k)</t>
+        </is>
+      </c>
       <c r="K19" s="168" t="n"/>
       <c r="L19" s="168" t="n"/>
       <c r="M19" s="168" t="n"/>
@@ -6980,13 +7087,10 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:J14"/>
-  <mergeCells count="8">
-    <mergeCell ref="B19:J19"/>
+  <mergeCells count="5">
     <mergeCell ref="B20:J20"/>
-    <mergeCell ref="A17:J17"/>
     <mergeCell ref="B22:J22"/>
     <mergeCell ref="B23:J23"/>
-    <mergeCell ref="B18:J18"/>
     <mergeCell ref="B21:J21"/>
     <mergeCell ref="B24:J24"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs: fix revisionCodes.ts filename in Sprint 0 sheet + roadmap update
</commit_message>
<xml_diff>
--- a/RevisionGrade_Roadmap_UPDATED.xlsx
+++ b/RevisionGrade_Roadmap_UPDATED.xlsx
@@ -6736,7 +6736,7 @@
       </c>
       <c r="G17" s="95" t="inlineStr">
         <is>
-          <t>docs/errors/, lib/errors/failureCodes.ts</t>
+          <t>docs/errors/, lib/errors/revisionCodes.ts</t>
         </is>
       </c>
       <c r="H17" s="95" t="inlineStr">
@@ -6751,7 +6751,7 @@
       </c>
       <c r="J17" s="95" t="inlineStr">
         <is>
-          <t>lib/errors/failureCodes.ts, PACK_F_EXECUTION_CONTRACT.md</t>
+          <t>lib/errors/revisionCodes.ts, PACK_F_EXECUTION_CONTRACT.md</t>
         </is>
       </c>
       <c r="K17" s="168" t="n"/>

</xml_diff>

<commit_message>
docs: mark 2.5 Completed in xlsx, add Sprint 0 subtasks 2.5.a/b, update counts (7 completed)
</commit_message>
<xml_diff>
--- a/RevisionGrade_Roadmap_UPDATED.xlsx
+++ b/RevisionGrade_Roadmap_UPDATED.xlsx
@@ -435,7 +435,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="189">
+  <cellXfs count="190">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -996,6 +996,9 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1443,6 +1446,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8" ht="14.25" customHeight="1" s="96">
       <c r="A8" s="95" t="inlineStr">
         <is>
@@ -1450,6 +1454,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="14.25" customHeight="1" s="96">
       <c r="A10" s="95" t="inlineStr">
         <is>
@@ -1460,7 +1465,7 @@
     <row r="11" ht="14.25" customHeight="1" s="96">
       <c r="A11" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Completed: 6 items (1.1, 1.2, 2.1, 2.2, 2.3, 2.4)</t>
+          <t xml:space="preserve">  Completed: 7 items (1.1, 1.2, 2.1, 2.2, 2.3, 2.4, 2.5)</t>
         </is>
       </c>
     </row>
@@ -1492,6 +1497,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="14.25" customHeight="1" s="96">
       <c r="A17" s="95" t="inlineStr">
         <is>
@@ -1527,6 +1533,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="14.25" customHeight="1" s="96">
       <c r="A23" s="95" t="inlineStr">
         <is>
@@ -1576,6 +1583,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31" ht="14.25" customHeight="1" s="96">
       <c r="A31" s="95" t="inlineStr">
         <is>
@@ -1639,6 +1647,7 @@
         </is>
       </c>
     </row>
+    <row r="40"/>
     <row r="41" ht="14.25" customHeight="1" s="96">
       <c r="A41" s="95" t="inlineStr">
         <is>
@@ -1747,6 +1756,7 @@
         </is>
       </c>
     </row>
+    <row r="59"/>
     <row r="60" ht="14.25" customHeight="1" s="96">
       <c r="A60" s="95" t="inlineStr">
         <is>
@@ -1779,7 +1789,7 @@
     <row r="65" ht="14.25" customHeight="1" s="96">
       <c r="A65" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Sprint 0 (Phase 2): 13 atomic subtasks for 2.1-2.4 with Success/Test/Artifact</t>
+          <t xml:space="preserve">  Sprint 0 (Phase 2): 15 atomic subtasks for 2.1-2.5 with Success/Test/Artifact</t>
         </is>
       </c>
     </row>
@@ -1797,6 +1807,7 @@
         </is>
       </c>
     </row>
+    <row r="68"/>
     <row r="69" ht="14.25" customHeight="1" s="96">
       <c r="A69" s="95" t="inlineStr">
         <is>
@@ -1910,7 +1921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B2:J28"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="95" min="1" max="1"/>
@@ -1922,6 +1933,7 @@
     <col width="15" customWidth="1" style="95" min="7" max="7"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="36" customHeight="1" s="96">
       <c r="B2" s="98" t="inlineStr">
         <is>
@@ -1943,6 +1955,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="24" customHeight="1" s="96">
       <c r="B6" s="101" t="inlineStr">
         <is>
@@ -1950,6 +1963,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8" ht="24" customHeight="1" s="96">
       <c r="B8" s="102" t="inlineStr">
         <is>
@@ -2008,6 +2022,8 @@
         <v/>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12" ht="24" customHeight="1" s="96">
       <c r="B12" s="101" t="inlineStr">
         <is>
@@ -2015,6 +2031,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="24" customHeight="1" s="96">
       <c r="B14" s="114" t="inlineStr">
         <is>
@@ -2174,6 +2191,7 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="15" customHeight="1" s="96">
       <c r="B22" s="95" t="n"/>
     </row>
@@ -2217,7 +2235,7 @@
       </c>
       <c r="C27" s="124" t="inlineStr">
         <is>
-          <t>Governed execution board: 13 atomic subtasks for 2.1-2.4 with Success/Test/Artifact</t>
+          <t>Governed execution board: 15 atomic subtasks for 2.1-2.5 with Success/Test/Artifact</t>
         </is>
       </c>
     </row>
@@ -3157,7 +3175,7 @@
       <c r="E11" s="137" t="n"/>
       <c r="F11" s="147" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="G11" s="139" t="inlineStr">
@@ -3208,7 +3226,7 @@
       </c>
       <c r="Q11" s="140" t="inlineStr">
         <is>
-          <t>Gate checkpoint before proceeding to 2.6.</t>
+          <t>COMPLETED at 48aa4c9 (2026-03-19). Deterministic matrix: 5 success cases (single, multi-proposal, literary prose, dialogue, multi-paragraph), 3 failure cases (PARSE_ERROR, ANCHOR_MISS, OFFSET_CONFLICT). 9/9 ingest, 9/9 extract, 9/9 validate, 9/9 apply. Repeated-run byte identity: true. 3 archived evidence runs. Closure doc published.</t>
         </is>
       </c>
       <c r="R11" s="141" t="inlineStr">
@@ -6890,8 +6908,56 @@
       <c r="T19" s="168" t="n"/>
     </row>
     <row r="20" ht="36" customHeight="1" s="96">
-      <c r="A20" s="168" t="n"/>
-      <c r="B20" s="168" t="n"/>
+      <c r="A20" s="189" t="inlineStr">
+        <is>
+          <t>S0-Apply-Engine</t>
+        </is>
+      </c>
+      <c r="B20" s="95" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="C20" s="95" t="inlineStr">
+        <is>
+          <t>Stage Validation</t>
+        </is>
+      </c>
+      <c r="D20" s="95" t="inlineStr">
+        <is>
+          <t>2.5.a</t>
+        </is>
+      </c>
+      <c r="E20" s="95" t="inlineStr">
+        <is>
+          <t>Build deterministic stage-validation e2e harness</t>
+        </is>
+      </c>
+      <c r="F20" s="95" t="inlineStr">
+        <is>
+          <t>Tests / Harness</t>
+        </is>
+      </c>
+      <c r="G20" s="95" t="inlineStr">
+        <is>
+          <t>tests/anchors/stage-validation-e2e.test.ts</t>
+        </is>
+      </c>
+      <c r="H20" s="95" t="inlineStr">
+        <is>
+          <t>5 success cases + 3 failure cases. 9/9 ingest, 9/9 extract, 9/9 validate, 9/9 apply. All pass.</t>
+        </is>
+      </c>
+      <c r="I20" s="95" t="inlineStr">
+        <is>
+          <t>npm test -- tests/anchors/stage-validation-e2e.test.ts. Verify JSON: pass=true.</t>
+        </is>
+      </c>
+      <c r="J20" s="95" t="inlineStr">
+        <is>
+          <t>stage-validation-e2e.test.ts, pack25 JSON/MD reports</t>
+        </is>
+      </c>
       <c r="K20" s="168" t="n"/>
       <c r="L20" s="168" t="n"/>
       <c r="M20" s="168" t="n"/>
@@ -6904,8 +6970,56 @@
       <c r="T20" s="168" t="n"/>
     </row>
     <row r="21" ht="36" customHeight="1" s="96">
-      <c r="A21" s="168" t="n"/>
-      <c r="B21" s="168" t="n"/>
+      <c r="A21" s="189" t="inlineStr">
+        <is>
+          <t>S0-Apply-Engine</t>
+        </is>
+      </c>
+      <c r="B21" s="95" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="C21" s="95" t="inlineStr">
+        <is>
+          <t>Stage Validation</t>
+        </is>
+      </c>
+      <c r="D21" s="95" t="inlineStr">
+        <is>
+          <t>2.5.b</t>
+        </is>
+      </c>
+      <c r="E21" s="95" t="inlineStr">
+        <is>
+          <t>Repeated-run byte identity proof + evidence archival</t>
+        </is>
+      </c>
+      <c r="F21" s="95" t="inlineStr">
+        <is>
+          <t>Tests / Evidence</t>
+        </is>
+      </c>
+      <c r="G21" s="95" t="inlineStr">
+        <is>
+          <t>docs/operations/evidence/runs/</t>
+        </is>
+      </c>
+      <c r="H21" s="95" t="inlineStr">
+        <is>
+          <t>repeated_run_identity_passed=true for all cases. Pipeline-identity byte-identical across runs. 3 evidence runs archived.</t>
+        </is>
+      </c>
+      <c r="I21" s="95" t="inlineStr">
+        <is>
+          <t>Run harness with PACK_25_REPORT_DIR. Verify JSON: repeated_run_identity_passed=true.</t>
+        </is>
+      </c>
+      <c r="J21" s="95" t="inlineStr">
+        <is>
+          <t>3 archived evidence directories under docs/operations/evidence/runs/</t>
+        </is>
+      </c>
       <c r="K21" s="168" t="n"/>
       <c r="L21" s="168" t="n"/>
       <c r="M21" s="168" t="n"/>
@@ -7087,11 +7201,9 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:J14"/>
-  <mergeCells count="5">
-    <mergeCell ref="B20:J20"/>
+  <mergeCells count="3">
     <mergeCell ref="B22:J22"/>
     <mergeCell ref="B23:J23"/>
-    <mergeCell ref="B21:J21"/>
     <mergeCell ref="B24:J24"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
roadmap: mark Phase 2.6 Completed, add Sprint 0 subtasks 2.6.a/b/c, update README (8 completed)
</commit_message>
<xml_diff>
--- a/RevisionGrade_Roadmap_UPDATED.xlsx
+++ b/RevisionGrade_Roadmap_UPDATED.xlsx
@@ -1398,7 +1398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A83"/>
+  <dimension ref="A1:A85"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="133.88" customWidth="1" style="95" min="1" max="1"/>
@@ -1446,7 +1446,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="14.25" customHeight="1" s="96">
       <c r="A8" s="95" t="inlineStr">
         <is>
@@ -1454,7 +1453,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="14.25" customHeight="1" s="96">
       <c r="A10" s="95" t="inlineStr">
         <is>
@@ -1465,7 +1463,7 @@
     <row r="11" ht="14.25" customHeight="1" s="96">
       <c r="A11" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Completed: 7 items (1.1, 1.2, 2.1, 2.2, 2.3, 2.4, 2.5)</t>
+          <t xml:space="preserve">  Completed: 8 items (1.1, 1.2, 2.1, 2.2, 2.3, 2.4, 2.5, 2.6)</t>
         </is>
       </c>
     </row>
@@ -1479,7 +1477,7 @@
     <row r="13" ht="14.25" customHeight="1" s="96">
       <c r="A13" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Next: 9 items</t>
+          <t xml:space="preserve">  Next: 8 items</t>
         </is>
       </c>
     </row>
@@ -1497,7 +1495,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="14.25" customHeight="1" s="96">
       <c r="A17" s="95" t="inlineStr">
         <is>
@@ -1533,7 +1530,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="14.25" customHeight="1" s="96">
       <c r="A23" s="95" t="inlineStr">
         <is>
@@ -1583,7 +1579,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31" ht="14.25" customHeight="1" s="96">
       <c r="A31" s="95" t="inlineStr">
         <is>
@@ -1634,24 +1629,30 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="95" t="inlineStr">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Stage Validation (2.5): COMPLETED &amp; VERIFIED (8 cases: 5 success + 3 failure, byte-identical repeat runs, 48aa4c9, 2026-03-19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="14.25" customHeight="1" s="96">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A6 Report Credibility (2.6): COMPLETED (rubric + confidence + provenance, 5 tests + evidence run, 0b0b657, 2026-03-19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="95" t="inlineStr">
         <is>
           <t xml:space="preserve">  Canon Integration (Phase 0): NEXT</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="14.25" customHeight="1" s="96">
-      <c r="A39" s="95" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Trust &amp; Quality Uplift: NEXT IN QUEUE</t>
-        </is>
-      </c>
-    </row>
-    <row r="40"/>
     <row r="41" ht="14.25" customHeight="1" s="96">
       <c r="A41" s="95" t="inlineStr">
         <is>
-          <t>---</t>
+          <t xml:space="preserve">  Trust &amp; Quality Uplift: NEXT IN QUEUE</t>
         </is>
       </c>
     </row>
@@ -1659,108 +1660,108 @@
     <row r="43" ht="14.25" customHeight="1" s="96">
       <c r="A43" s="95" t="inlineStr">
         <is>
-          <t>Three-Layer Execution Structure</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="14.25" customHeight="1" s="96">
-      <c r="A44" s="95" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Layer 1 — Roadmap: direction + sequencing (this workbook)</t>
-        </is>
-      </c>
-    </row>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="14.25" customHeight="1" s="96"/>
     <row r="45">
       <c r="A45" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Layer 2 — Sprint: atomic subtasks with verification (Sprint 0 sheet)</t>
+          <t>Three-Layer Execution Structure</t>
         </is>
       </c>
     </row>
     <row r="46" ht="14.25" customHeight="1" s="96">
       <c r="A46" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Layer 3 — Authority: canon enforcement at runtime (Phase 0 items)</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="14.25" customHeight="1" s="96"/>
+          <t xml:space="preserve">  Layer 1 — Roadmap: direction + sequencing (this workbook)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="14.25" customHeight="1" s="96">
+      <c r="A47" s="95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Layer 2 — Sprint: atomic subtasks with verification (Sprint 0 sheet)</t>
+        </is>
+      </c>
+    </row>
     <row r="48" ht="14.25" customHeight="1" s="96">
       <c r="A48" s="95" t="inlineStr">
         <is>
-          <t>Governance Model</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="14.25" customHeight="1" s="96">
-      <c r="A49" s="95" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Every roadmap item has: Success Criteria, Test Method, Canon Reference</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">  Layer 3 — Authority: canon enforcement at runtime (Phase 0 items)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="14.25" customHeight="1" s="96"/>
     <row r="50" ht="14.25" customHeight="1" s="96">
       <c r="A50" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Every sprint subtask has: Success Criteria, Test Method, Output Artifact</t>
+          <t>Governance Model</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Definition of done: "This passed its defined success test" — not "I think this is done"</t>
+          <t xml:space="preserve">  Every roadmap item has: Success Criteria, Test Method, Canon Reference</t>
         </is>
       </c>
     </row>
     <row r="52" ht="14.25" customHeight="1" s="96">
       <c r="A52" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Canon compliance check required before any phase can be marked verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="14.25" customHeight="1" s="96"/>
+          <t xml:space="preserve">  Every sprint subtask has: Success Criteria, Test Method, Output Artifact</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="14.25" customHeight="1" s="96">
+      <c r="A53" s="95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Definition of done: "This passed its defined success test" — not "I think this is done"</t>
+        </is>
+      </c>
+    </row>
     <row r="54" ht="14.25" customHeight="1" s="96">
       <c r="A54" s="95" t="inlineStr">
         <is>
-          <t>Active Gates</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="14.25" customHeight="1" s="96">
-      <c r="A55" s="95" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2.1 DB Verification: phase21-db-verification.sql must pass before 2.2 begins</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">  Canon compliance check required before any phase can be marked verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="14.25" customHeight="1" s="96"/>
     <row r="56" ht="14.25" customHeight="1" s="96">
       <c r="A56" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Canon Gate (Pass 1.5): Must execute before results surface to users</t>
+          <t>Active Gates</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Two-AI Independence: Pass 2 must never receive Pass 1 outputs</t>
+          <t xml:space="preserve">  2.1 DB Verification: phase21-db-verification.sql must pass before 2.2 begins</t>
         </is>
       </c>
     </row>
     <row r="58" ht="14.25" customHeight="1" s="96">
       <c r="A58" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Audit Spine: Append-only, hash-chained, no DELETE/UPDATE, 7-year retention</t>
-        </is>
-      </c>
-    </row>
-    <row r="59"/>
+          <t xml:space="preserve">  Canon Gate (Pass 1.5): Must execute before results surface to users</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Two-AI Independence: Pass 2 must never receive Pass 1 outputs</t>
+        </is>
+      </c>
+    </row>
     <row r="60" ht="14.25" customHeight="1" s="96">
       <c r="A60" s="95" t="inlineStr">
         <is>
-          <t>---</t>
+          <t xml:space="preserve">  Audit Spine: Append-only, hash-chained, no DELETE/UPDATE, 7-year retention</t>
         </is>
       </c>
     </row>
@@ -1768,50 +1769,50 @@
     <row r="62" ht="14.25" customHeight="1" s="96">
       <c r="A62" s="95" t="inlineStr">
         <is>
-          <t>Workbook Sheets</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="14.25" customHeight="1" s="96">
-      <c r="A63" s="95" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Overview: Dashboard with KPI cards and phase progress</t>
-        </is>
-      </c>
-    </row>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="14.25" customHeight="1" s="96"/>
     <row r="64" ht="14.25" customHeight="1" s="96">
       <c r="A64" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Roadmap: Full 44-item sequential tracker with all PM fields + Canon Reference</t>
+          <t>Workbook Sheets</t>
         </is>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1" s="96">
       <c r="A65" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Sprint 0 (Phase 2): 15 atomic subtasks for 2.1-2.5 with Success/Test/Artifact</t>
+          <t xml:space="preserve">  Overview: Dashboard with KPI cards and phase progress</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Immediate Priorities: The 'next three' critical deliverables</t>
+          <t xml:space="preserve">  Roadmap: Full 44-item sequential tracker with all PM fields + Canon Reference</t>
         </is>
       </c>
     </row>
     <row r="67" ht="14.25" customHeight="1" s="96">
       <c r="A67" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Canon Reference: Authority chain, numeric constants, 10 non-negotiable governance rules</t>
-        </is>
-      </c>
-    </row>
-    <row r="68"/>
+          <t xml:space="preserve">  Sprint 0 (Phase 2): 18 atomic subtasks for 2.1-2.6 with Success/Test/Artifact</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Immediate Priorities: The 'next three' critical deliverables</t>
+        </is>
+      </c>
+    </row>
     <row r="69" ht="14.25" customHeight="1" s="96">
       <c r="A69" s="95" t="inlineStr">
         <is>
-          <t>---</t>
+          <t xml:space="preserve">  Canon Reference: Authority chain, numeric constants, 10 non-negotiable governance rules</t>
         </is>
       </c>
     </row>
@@ -1819,89 +1820,97 @@
     <row r="71" ht="14.25" customHeight="1" s="96">
       <c r="A71" s="95" t="inlineStr">
         <is>
-          <t>Canon Document Sources (20 documents integrated)</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="14.25" customHeight="1" s="96">
-      <c r="A72" s="95" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Volume I — WAVE Revision Guide Canon (62 waves, 3 tsunamis, 10 execution rules)</t>
-        </is>
-      </c>
-    </row>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="14.25" customHeight="1" s="96"/>
     <row r="73" ht="14.25" customHeight="1" s="96">
       <c r="A73" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume II — Story Evaluation Criteria (13 criteria, 10 diagnostic patterns)</t>
+          <t>Canon Document Sources (20 documents integrated)</t>
         </is>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1" s="96">
       <c r="A74" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume II-A — Operational Schema (weights, gates, JSON envelope, Supabase tables)</t>
+          <t xml:space="preserve">  Volume I — WAVE Revision Guide Canon (62 waves, 3 tsunamis, 10 execution rules)</t>
         </is>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1" s="96">
       <c r="A75" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume III — Platform Governance Canon (5 doctrines, 3-layer editorial intelligence)</t>
+          <t xml:space="preserve">  Volume II — Story Evaluation Criteria (13 criteria, 10 diagnostic patterns)</t>
         </is>
       </c>
     </row>
     <row r="76" ht="14.25" customHeight="1" s="96">
       <c r="A76" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume III — Tools &amp; Implementation Systems (schemas, prompts, adapters)</t>
+          <t xml:space="preserve">  Volume II-A — Operational Schema (weights, gates, JSON envelope, Supabase tables)</t>
         </is>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1" s="96">
       <c r="A77" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume III — Operational Specification (thresholds, routing, 7-stage pipeline)</t>
+          <t xml:space="preserve">  Volume III — Platform Governance Canon (5 doctrines, 3-layer editorial intelligence)</t>
         </is>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1" s="96">
       <c r="A78" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume IV — AI Governance Canon (3-layer authority, 7 protection systems)</t>
+          <t xml:space="preserve">  Volume III — Tools &amp; Implementation Systems (schemas, prompts, adapters)</t>
         </is>
       </c>
     </row>
     <row r="79" ht="14.25" customHeight="1" s="96">
       <c r="A79" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume V — Execution Architecture (AEP 6-step flow, Trifecta, chunking, reliability)</t>
+          <t xml:space="preserve">  Volume III — Operational Specification (thresholds, routing, 7-stage pipeline)</t>
         </is>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1" s="96">
       <c r="A80" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Canon III — Lessons of the Living System (8 governing laws)</t>
+          <t xml:space="preserve">  Volume IV — AI Governance Canon (3-layer authority, 7 protection systems)</t>
         </is>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1" s="96">
       <c r="A81" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Canon Assembly Matrix (RCAM v2.0, 24 source docs, 5 matrix rules)</t>
+          <t xml:space="preserve">  Volume V — Execution Architecture (AEP 6-step flow, Trifecta, chunking, reliability)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Canon Doctrine Registry (77 doctrine units, 6 governance rules)</t>
+          <t xml:space="preserve">  Canon III — Lessons of the Living System (8 governing laws)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Canon Assembly Matrix (RCAM v2.0, 24 source docs, 5 matrix rules)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Canon Doctrine Registry (77 doctrine units, 6 governance rules)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="95" t="inlineStr">
         <is>
           <t xml:space="preserve">  + 9 supporting/variant documents (txt, md formats)</t>
         </is>
@@ -1921,7 +1930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="B2:J28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="95" min="1" max="1"/>
@@ -1933,7 +1942,6 @@
     <col width="15" customWidth="1" style="95" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="36" customHeight="1" s="96">
       <c r="B2" s="98" t="inlineStr">
         <is>
@@ -1955,7 +1963,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="24" customHeight="1" s="96">
       <c r="B6" s="101" t="inlineStr">
         <is>
@@ -1963,7 +1970,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="24" customHeight="1" s="96">
       <c r="B8" s="102" t="inlineStr">
         <is>
@@ -2022,8 +2028,6 @@
         <v/>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12" ht="24" customHeight="1" s="96">
       <c r="B12" s="101" t="inlineStr">
         <is>
@@ -2031,7 +2035,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="24" customHeight="1" s="96">
       <c r="B14" s="114" t="inlineStr">
         <is>
@@ -2191,7 +2194,6 @@
         <v/>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="15" customHeight="1" s="96">
       <c r="B22" s="95" t="n"/>
     </row>
@@ -3255,7 +3257,7 @@
       <c r="E12" s="143" t="n"/>
       <c r="F12" s="147" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="G12" s="148" t="inlineStr">
@@ -3298,7 +3300,11 @@
           <t>Rubric breakdown, score explanations, confidence, and provenance visible on report. Zero recomputation on read.</t>
         </is>
       </c>
-      <c r="O12" s="145" t="n"/>
+      <c r="O12" s="145" t="inlineStr">
+        <is>
+          <t>4 unit tests (credibility, missing-refs, phantom-anchor, confidence-richness) + 1 artifact output test (JSON+MD write verification) + evidence run validation</t>
+        </is>
+      </c>
       <c r="P12" s="145" t="inlineStr">
         <is>
           <t>No</t>
@@ -3306,7 +3312,7 @@
       </c>
       <c r="Q12" s="145" t="inlineStr">
         <is>
-          <t>Partially implemented. Roadmap Item 1 from narrative. Must close on top of Gate A5.</t>
+          <t>COMPLETED at 0b0b657 (2026-03-19). Implementation: types.ts, buildA6Report.ts, confidence.ts, provenance.ts, validateA6Report.ts, writeA6Artifacts.ts, run-a6-evidence.ts. Tests: a6-report-credibility.test.ts (4 cases: rubric+confidence+provenance, missing-evidence-refs, phantom-anchor, confidence-richness), a6-artifact-output.test.ts (JSON+MD artifact write). Evidence: 2 criteria (narrative_cohesion 8.5/10, tone_consistency 8.9/10), overall 8.7, confidence 0.9, 2 provenance entries, all anchors resolve. Validation: all_criteria_have_reasoning=true, all_reasoning_has_evidence=true, all_anchors_resolve=true, confidence_is_derived=true. Closure doc at a85512a (empty placeholder — needs content backfill).</t>
         </is>
       </c>
       <c r="R12" s="141" t="inlineStr">
@@ -5960,7 +5966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:T29"/>
+  <dimension ref="A1:T32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="95" min="1" max="1"/>
@@ -7032,142 +7038,238 @@
       <c r="T21" s="168" t="n"/>
     </row>
     <row r="22" ht="36" customHeight="1" s="96">
-      <c r="A22" s="101" t="inlineStr">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>S0-Apply-Engine</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>A6 Report Credibility</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2.6.a</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Build A6 report: types, buildA6Report, confidence, provenance, validateA6Report, writeA6Artifacts</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>lib/evaluation/a6/</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>buildA6Report produces valid rubric + confidence + provenance; validateA6Report enforces invariants</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>4 unit tests in a6-report-credibility.test.ts (rubric, missing-refs, phantom-anchor, confidence-richness)</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>lib/evaluation/a6/*.ts (6 modules), a6_report.json, a6_validation_summary.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="36" customHeight="1" s="96">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>S0-Apply-Engine</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>A6 Report Credibility</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2.6.b</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Evidence run: run-a6-evidence.ts + artifact output (JSON+MD) + validation summary</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Tests / Evidence</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>scripts/a6/, tests/evaluation/, docs/operations/evidence/runs/</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Evidence artifacts generated, all invariants pass, failure cases (missing-refs, phantom-anchor) tested</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>a6-artifact-output.test.ts (JSON+MD write) + run-a6-evidence.ts execution</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>a6_report.json, a6_report.md, a6_validation_summary.json, metadata.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="36" customHeight="1" s="96">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>S0-Apply-Engine</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>A6 Report Credibility</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2.6.c</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Closure documentation + ChatGPT verification audit</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>PHASE_2_6_A6_REPORT_CREDIBILITY_CLOSURE.md</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Closure doc contains: spec compliance, evidence links, invariant proof, offset analysis, open items</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Manual review: closure doc completeness check against GATE_A6_REPORT_CREDIBILITY.md spec</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>PHASE_2_6_A6_REPORT_CREDIBILITY_CLOSURE.md (needs content backfill — committed empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="135.75" customHeight="1" s="96">
+      <c r="A25" s="101" t="inlineStr">
         <is>
           <t>EXECUTION GOVERNANCE NOTES</t>
         </is>
       </c>
-      <c r="B22" s="95" t="n"/>
-      <c r="K22" s="168" t="n"/>
-      <c r="L22" s="168" t="n"/>
-      <c r="M22" s="168" t="n"/>
-      <c r="N22" s="168" t="n"/>
-      <c r="O22" s="168" t="n"/>
-      <c r="P22" s="168" t="n"/>
-      <c r="Q22" s="168" t="n"/>
-      <c r="R22" s="168" t="n"/>
-      <c r="S22" s="168" t="n"/>
-      <c r="T22" s="168" t="n"/>
-    </row>
-    <row r="23" ht="36" customHeight="1" s="96">
-      <c r="A23" s="172" t="inlineStr">
-        <is>
-          <t>Current State</t>
-        </is>
-      </c>
-      <c r="B23" s="173" t="inlineStr">
-        <is>
-          <t>Roadmap (strategic) + Sprint (operational) + Verification (truth). Three-layer execution structure.</t>
-        </is>
-      </c>
-      <c r="C23" s="170" t="n"/>
-      <c r="D23" s="170" t="n"/>
-      <c r="E23" s="170" t="n"/>
-      <c r="F23" s="170" t="n"/>
-      <c r="G23" s="170" t="n"/>
-      <c r="H23" s="170" t="n"/>
-      <c r="I23" s="170" t="n"/>
-      <c r="J23" s="170" t="n"/>
-      <c r="K23" s="168" t="n"/>
-      <c r="L23" s="168" t="n"/>
-      <c r="M23" s="168" t="n"/>
-      <c r="N23" s="168" t="n"/>
-      <c r="O23" s="168" t="n"/>
-      <c r="P23" s="168" t="n"/>
-      <c r="Q23" s="168" t="n"/>
-      <c r="R23" s="168" t="n"/>
-      <c r="S23" s="168" t="n"/>
-      <c r="T23" s="168" t="n"/>
-    </row>
-    <row r="24" ht="36" customHeight="1" s="96">
-      <c r="A24" s="172" t="inlineStr">
-        <is>
-          <t>Core Principle</t>
-        </is>
-      </c>
-      <c r="B24" s="173" t="inlineStr">
-        <is>
-          <t>Eliminate "I think this is done." Replace with "This passed its defined success test." Every row has provable completion.</t>
-        </is>
-      </c>
-      <c r="C24" s="170" t="n"/>
-      <c r="D24" s="170" t="n"/>
-      <c r="E24" s="170" t="n"/>
-      <c r="F24" s="170" t="n"/>
-      <c r="G24" s="170" t="n"/>
-      <c r="H24" s="170" t="n"/>
-      <c r="I24" s="170" t="n"/>
-      <c r="J24" s="170" t="n"/>
-    </row>
-    <row r="25" ht="135.75" customHeight="1" s="96">
-      <c r="A25" s="172" t="inlineStr">
-        <is>
-          <t>Critical Path</t>
-        </is>
-      </c>
-      <c r="B25" s="173" t="inlineStr">
-        <is>
-          <t>2.1 → 2.2 → 2.3 → 2.4. Do NOT parallelize. Each depends on the prior being VERIFIED, not just coded.</t>
-        </is>
-      </c>
-      <c r="C25" s="174" t="n"/>
-      <c r="D25" s="174" t="n"/>
-      <c r="E25" s="174" t="n"/>
-      <c r="F25" s="174" t="n"/>
-      <c r="G25" s="174" t="n"/>
-      <c r="H25" s="174" t="n"/>
-      <c r="I25" s="174" t="n"/>
-      <c r="J25" s="174" t="n"/>
+      <c r="B25" s="95" t="n"/>
+      <c r="K25" s="168" t="n"/>
+      <c r="L25" s="168" t="n"/>
+      <c r="M25" s="168" t="n"/>
+      <c r="N25" s="168" t="n"/>
+      <c r="O25" s="168" t="n"/>
+      <c r="P25" s="168" t="n"/>
+      <c r="Q25" s="168" t="n"/>
+      <c r="R25" s="168" t="n"/>
+      <c r="S25" s="168" t="n"/>
+      <c r="T25" s="168" t="n"/>
     </row>
     <row r="26" ht="225" customHeight="1" s="96">
       <c r="A26" s="172" t="inlineStr">
         <is>
-          <t>2.3 Is The Product</t>
+          <t>Current State</t>
         </is>
       </c>
       <c r="B26" s="173" t="inlineStr">
         <is>
-          <t>The apply engine is the product. Everything else — UI, reports, packaging — is presentation. If 2.3 is deterministic, idempotent, and precise, you win. If not, everything collapses.</t>
-        </is>
-      </c>
-      <c r="C26" s="174" t="n"/>
-      <c r="D26" s="174" t="n"/>
-      <c r="E26" s="174" t="n"/>
-      <c r="F26" s="174" t="n"/>
-      <c r="G26" s="174" t="n"/>
-      <c r="H26" s="174" t="n"/>
-      <c r="I26" s="174" t="n"/>
-      <c r="J26" s="174" t="n"/>
+          <t>Roadmap (strategic) + Sprint (operational) + Verification (truth). Three-layer execution structure.</t>
+        </is>
+      </c>
+      <c r="C26" s="170" t="n"/>
+      <c r="D26" s="170" t="n"/>
+      <c r="E26" s="170" t="n"/>
+      <c r="F26" s="170" t="n"/>
+      <c r="G26" s="170" t="n"/>
+      <c r="H26" s="170" t="n"/>
+      <c r="I26" s="170" t="n"/>
+      <c r="J26" s="170" t="n"/>
+      <c r="K26" s="168" t="n"/>
+      <c r="L26" s="168" t="n"/>
+      <c r="M26" s="168" t="n"/>
+      <c r="N26" s="168" t="n"/>
+      <c r="O26" s="168" t="n"/>
+      <c r="P26" s="168" t="n"/>
+      <c r="Q26" s="168" t="n"/>
+      <c r="R26" s="168" t="n"/>
+      <c r="S26" s="168" t="n"/>
+      <c r="T26" s="168" t="n"/>
     </row>
     <row r="27" ht="202.5" customHeight="1" s="96">
       <c r="A27" s="172" t="inlineStr">
         <is>
-          <t>When 2.3 Fails</t>
+          <t>Core Principle</t>
         </is>
       </c>
       <c r="B27" s="173" t="inlineStr">
         <is>
-          <t>Do NOT patch. Do NOT add hacks. Log everything → classify failures (2.4) → refine determinism. This is the discipline that separates a system from a tool.</t>
-        </is>
-      </c>
-      <c r="C27" s="174" t="n"/>
-      <c r="D27" s="174" t="n"/>
-      <c r="E27" s="174" t="n"/>
-      <c r="F27" s="174" t="n"/>
-      <c r="G27" s="174" t="n"/>
-      <c r="H27" s="174" t="n"/>
-      <c r="I27" s="174" t="n"/>
-      <c r="J27" s="174" t="n"/>
+          <t>Eliminate "I think this is done." Replace with "This passed its defined success test." Every row has provable completion.</t>
+        </is>
+      </c>
+      <c r="C27" s="170" t="n"/>
+      <c r="D27" s="170" t="n"/>
+      <c r="E27" s="170" t="n"/>
+      <c r="F27" s="170" t="n"/>
+      <c r="G27" s="170" t="n"/>
+      <c r="H27" s="170" t="n"/>
+      <c r="I27" s="170" t="n"/>
+      <c r="J27" s="170" t="n"/>
     </row>
     <row r="28" ht="191.25" customHeight="1" s="96">
       <c r="A28" s="172" t="inlineStr">
         <is>
-          <t>Scope Discipline</t>
+          <t>Critical Path</t>
         </is>
       </c>
       <c r="B28" s="173" t="inlineStr">
         <is>
-          <t>Do NOT expand scope. Do NOT add features. Finish 2.1 VERIFIED → 2.2 VERIFIED → 2.3 VERIFIED → 2.4 VERIFIED. Then and only then move forward.</t>
+          <t>2.1 → 2.2 → 2.3 → 2.4. Do NOT parallelize. Each depends on the prior being VERIFIED, not just coded.</t>
         </is>
       </c>
       <c r="C28" s="174" t="n"/>
@@ -7182,12 +7284,12 @@
     <row r="29" ht="314.25" customHeight="1" s="96">
       <c r="A29" s="172" t="inlineStr">
         <is>
-          <t>2.1 VERIFIED (2026-03-18). Code complete + tests pass + DB verification 6/6 gates passed on target DB. 21 anchored rows verified — deterministic slice contract holds. Data remediation: 2 manuscript_versions backfilled (raw_text from file_url), 15 anchor offsets recomputed. GATE CLEARED → 2.2 may proceed.</t>
+          <t>2.3 Is The Product</t>
         </is>
       </c>
       <c r="B29" s="173" t="inlineStr">
         <is>
-          <t>2.1 CODE COMPLETE + TEST VERIFIED. DB rollout pending. SQL verification pack created (phase21-db-verification.sql). Runbook at tests/anchors/PHASE21_DB_VERIFICATION_RUNBOOK.md. GATE: DB verification must pass before 2.2 begins.</t>
+          <t>The apply engine is the product. Everything else — UI, reports, packaging — is presentation. If 2.3 is deterministic, idempotent, and precise, you win. If not, everything collapses.</t>
         </is>
       </c>
       <c r="C29" s="174" t="n"/>
@@ -7199,11 +7301,71 @@
       <c r="I29" s="174" t="n"/>
       <c r="J29" s="174" t="n"/>
     </row>
+    <row r="30">
+      <c r="A30" s="172" t="inlineStr">
+        <is>
+          <t>When 2.3 Fails</t>
+        </is>
+      </c>
+      <c r="B30" s="173" t="inlineStr">
+        <is>
+          <t>Do NOT patch. Do NOT add hacks. Log everything → classify failures (2.4) → refine determinism. This is the discipline that separates a system from a tool.</t>
+        </is>
+      </c>
+      <c r="C30" s="174" t="n"/>
+      <c r="D30" s="174" t="n"/>
+      <c r="E30" s="174" t="n"/>
+      <c r="F30" s="174" t="n"/>
+      <c r="G30" s="174" t="n"/>
+      <c r="H30" s="174" t="n"/>
+      <c r="I30" s="174" t="n"/>
+      <c r="J30" s="174" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="172" t="inlineStr">
+        <is>
+          <t>Scope Discipline</t>
+        </is>
+      </c>
+      <c r="B31" s="173" t="inlineStr">
+        <is>
+          <t>Do NOT expand scope. Do NOT add features. Finish 2.1 VERIFIED → 2.2 VERIFIED → 2.3 VERIFIED → 2.4 VERIFIED. Then and only then move forward.</t>
+        </is>
+      </c>
+      <c r="C31" s="174" t="n"/>
+      <c r="D31" s="174" t="n"/>
+      <c r="E31" s="174" t="n"/>
+      <c r="F31" s="174" t="n"/>
+      <c r="G31" s="174" t="n"/>
+      <c r="H31" s="174" t="n"/>
+      <c r="I31" s="174" t="n"/>
+      <c r="J31" s="174" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="172" t="inlineStr">
+        <is>
+          <t>2.1 VERIFIED (2026-03-18). Code complete + tests pass + DB verification 6/6 gates passed on target DB. 21 anchored rows verified — deterministic slice contract holds. Data remediation: 2 manuscript_versions backfilled (raw_text from file_url), 15 anchor offsets recomputed. GATE CLEARED → 2.2 may proceed.</t>
+        </is>
+      </c>
+      <c r="B32" s="173" t="inlineStr">
+        <is>
+          <t>2.1 CODE COMPLETE + TEST VERIFIED. DB rollout pending. SQL verification pack created (phase21-db-verification.sql). Runbook at tests/anchors/PHASE21_DB_VERIFICATION_RUNBOOK.md. GATE: DB verification must pass before 2.2 begins.</t>
+        </is>
+      </c>
+      <c r="C32" s="174" t="n"/>
+      <c r="D32" s="174" t="n"/>
+      <c r="E32" s="174" t="n"/>
+      <c r="F32" s="174" t="n"/>
+      <c r="G32" s="174" t="n"/>
+      <c r="H32" s="174" t="n"/>
+      <c r="I32" s="174" t="n"/>
+      <c r="J32" s="174" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J14"/>
   <mergeCells count="3">
+    <mergeCell ref="B23:J23"/>
     <mergeCell ref="B22:J22"/>
-    <mergeCell ref="B23:J23"/>
     <mergeCell ref="B24:J24"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
roadmap: fix Sprint 0 2.6 subtasks (unmerge + populate), upgrade 2.6 to VERIFIED, ref 38d9c19
</commit_message>
<xml_diff>
--- a/RevisionGrade_Roadmap_UPDATED.xlsx
+++ b/RevisionGrade_Roadmap_UPDATED.xlsx
@@ -1629,16 +1629,16 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="95" t="inlineStr">
         <is>
           <t xml:space="preserve">  Stage Validation (2.5): COMPLETED &amp; VERIFIED (8 cases: 5 success + 3 failure, byte-identical repeat runs, 48aa4c9, 2026-03-19)</t>
         </is>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1" s="96">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  A6 Report Credibility (2.6): COMPLETED (rubric + confidence + provenance, 5 tests + evidence run, 0b0b657, 2026-03-19)</t>
+      <c r="A39" s="95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A6 Report Credibility (2.6): COMPLETED &amp; VERIFIED (rubric + confidence + provenance, 5 tests + evidence run, offset-consistent, 38d9c19, 2026-03-19)</t>
         </is>
       </c>
     </row>
@@ -3312,7 +3312,7 @@
       </c>
       <c r="Q12" s="145" t="inlineStr">
         <is>
-          <t>COMPLETED at 0b0b657 (2026-03-19). Implementation: types.ts, buildA6Report.ts, confidence.ts, provenance.ts, validateA6Report.ts, writeA6Artifacts.ts, run-a6-evidence.ts. Tests: a6-report-credibility.test.ts (4 cases: rubric+confidence+provenance, missing-evidence-refs, phantom-anchor, confidence-richness), a6-artifact-output.test.ts (JSON+MD artifact write). Evidence: 2 criteria (narrative_cohesion 8.5/10, tone_consistency 8.9/10), overall 8.7, confidence 0.9, 2 provenance entries, all anchors resolve. Validation: all_criteria_have_reasoning=true, all_reasoning_has_evidence=true, all_anchors_resolve=true, confidence_is_derived=true. Closure doc at a85512a (empty placeholder — needs content backfill).</t>
+          <t>COMPLETED at 0b0b657, verified at 38d9c19 (2026-03-19). 6 modules: types.ts, buildA6Report.ts, confidence.ts, provenance.ts, validateA6Report.ts, writeA6Artifacts.ts. 5 tests: rubric+confidence+provenance, missing-evidence-refs, phantom-anchor, confidence-richness, artifact-output. Evidence: narrative_cohesion 8.5/10, tone_consistency 8.9/10, overall 8.7, confidence 0.9, 2 provenance entries, offsets [4,22) [43,86) consistent. All invariants pass. Closure doc: 151 lines, fully populated.</t>
         </is>
       </c>
       <c r="R12" s="141" t="inlineStr">
@@ -7038,12 +7038,12 @@
       <c r="T21" s="168" t="n"/>
     </row>
     <row r="22" ht="36" customHeight="1" s="96">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="95" t="inlineStr">
         <is>
           <t>S0-Apply-Engine</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="95" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
@@ -7090,12 +7090,12 @@
       </c>
     </row>
     <row r="23" ht="36" customHeight="1" s="96">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="95" t="inlineStr">
         <is>
           <t>S0-Apply-Engine</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="95" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
@@ -7112,7 +7112,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Evidence run: run-a6-evidence.ts + artifact output (JSON+MD) + validation summary</t>
+          <t>Evidence run + artifact output (JSON+MD) + validation summary</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -7142,12 +7142,12 @@
       </c>
     </row>
     <row r="24" ht="36" customHeight="1" s="96">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="95" t="inlineStr">
         <is>
           <t>S0-Apply-Engine</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="95" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
@@ -7164,7 +7164,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Closure documentation + ChatGPT verification audit</t>
+          <t>Closure documentation + offset audit + ChatGPT verification</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -7179,17 +7179,17 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Closure doc contains: spec compliance, evidence links, invariant proof, offset analysis, open items</t>
+          <t>Closure doc populated (151 lines), spec compliance verified, offset consistency confirmed [43,86)</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Manual review: closure doc completeness check against GATE_A6_REPORT_CREDIBILITY.md spec</t>
+          <t>Manual review: closure doc completeness, offset consistency, 5/5 tests green post-fix (38d9c19)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>PHASE_2_6_A6_REPORT_CREDIBILITY_CLOSURE.md (needs content backfill — committed empty)</t>
+          <t>PHASE_2_6_A6_REPORT_CREDIBILITY_CLOSURE.md (populated at 38d9c19)</t>
         </is>
       </c>
     </row>
@@ -7363,11 +7363,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:J14"/>
-  <mergeCells count="3">
-    <mergeCell ref="B23:J23"/>
-    <mergeCell ref="B22:J22"/>
-    <mergeCell ref="B24:J24"/>
-  </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
roadmap: fix Sprint 0 2.6.c line count (151→214) to match actual closure doc on main
</commit_message>
<xml_diff>
--- a/RevisionGrade_Roadmap_UPDATED.xlsx
+++ b/RevisionGrade_Roadmap_UPDATED.xlsx
@@ -3312,7 +3312,7 @@
       </c>
       <c r="Q12" s="145" t="inlineStr">
         <is>
-          <t>COMPLETED at 0b0b657, verified at 38d9c19 (2026-03-19). 6 modules: types.ts, buildA6Report.ts, confidence.ts, provenance.ts, validateA6Report.ts, writeA6Artifacts.ts. 5 tests: rubric+confidence+provenance, missing-evidence-refs, phantom-anchor, confidence-richness, artifact-output. Evidence: narrative_cohesion 8.5/10, tone_consistency 8.9/10, overall 8.7, confidence 0.9, 2 provenance entries, offsets [4,22) [43,86) consistent. All invariants pass. Closure doc: 151 lines, fully populated.</t>
+          <t>COMPLETED at 0b0b657, verified at 38d9c19, closure doc landed at 66b84e4 (2026-03-19). 6 modules: types.ts, buildA6Report.ts, confidence.ts, provenance.ts, validateA6Report.ts, writeA6Artifacts.ts. 5 tests: rubric+confidence+provenance, missing-evidence-refs, phantom-anchor, confidence-richness, artifact-output. Evidence: narrative_cohesion 8.5/10, tone_consistency 8.9/10, overall 8.7, confidence 0.9, 2 provenance entries, offsets [4,22) [43,86) consistent. All invariants pass. Closure doc: 214 lines on main, fully populated.</t>
         </is>
       </c>
       <c r="R12" s="141" t="inlineStr">
@@ -7048,42 +7048,42 @@
           <t>2.6</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="95" t="inlineStr">
         <is>
           <t>A6 Report Credibility</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="95" t="inlineStr">
         <is>
           <t>2.6.a</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="95" t="inlineStr">
         <is>
           <t>Build A6 report: types, buildA6Report, confidence, provenance, validateA6Report, writeA6Artifacts</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F22" s="95" t="inlineStr">
         <is>
           <t>Backend</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G22" s="95" t="inlineStr">
         <is>
           <t>lib/evaluation/a6/</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H22" s="95" t="inlineStr">
         <is>
           <t>buildA6Report produces valid rubric + confidence + provenance; validateA6Report enforces invariants</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="I22" s="95" t="inlineStr">
         <is>
           <t>4 unit tests in a6-report-credibility.test.ts (rubric, missing-refs, phantom-anchor, confidence-richness)</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="J22" s="95" t="inlineStr">
         <is>
           <t>lib/evaluation/a6/*.ts (6 modules), a6_report.json, a6_validation_summary.json</t>
         </is>
@@ -7100,42 +7100,42 @@
           <t>2.6</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="95" t="inlineStr">
         <is>
           <t>A6 Report Credibility</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="95" t="inlineStr">
         <is>
           <t>2.6.b</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="95" t="inlineStr">
         <is>
           <t>Evidence run + artifact output (JSON+MD) + validation summary</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F23" s="95" t="inlineStr">
         <is>
           <t>Tests / Evidence</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" s="95" t="inlineStr">
         <is>
           <t>scripts/a6/, tests/evaluation/, docs/operations/evidence/runs/</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H23" s="95" t="inlineStr">
         <is>
           <t>Evidence artifacts generated, all invariants pass, failure cases (missing-refs, phantom-anchor) tested</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I23" s="95" t="inlineStr">
         <is>
           <t>a6-artifact-output.test.ts (JSON+MD write) + run-a6-evidence.ts execution</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="J23" s="95" t="inlineStr">
         <is>
           <t>a6_report.json, a6_report.md, a6_validation_summary.json, metadata.json</t>
         </is>
@@ -7152,44 +7152,44 @@
           <t>2.6</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="95" t="inlineStr">
         <is>
           <t>A6 Report Credibility</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="95" t="inlineStr">
         <is>
           <t>2.6.c</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="95" t="inlineStr">
         <is>
           <t>Closure documentation + offset audit + ChatGPT verification</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F24" s="95" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G24" s="95" t="inlineStr">
         <is>
           <t>PHASE_2_6_A6_REPORT_CREDIBILITY_CLOSURE.md</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Closure doc populated (151 lines), spec compliance verified, offset consistency confirmed [43,86)</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
+      <c r="H24" s="95" t="inlineStr">
+        <is>
+          <t>Closure doc populated (214 lines, 7559 bytes on main), spec compliance verified, offset consistency confirmed [43,86)</t>
+        </is>
+      </c>
+      <c r="I24" s="95" t="inlineStr">
         <is>
           <t>Manual review: closure doc completeness, offset consistency, 5/5 tests green post-fix (38d9c19)</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>PHASE_2_6_A6_REPORT_CREDIBILITY_CLOSURE.md (populated at 38d9c19)</t>
+      <c r="J24" s="95" t="inlineStr">
+        <is>
+          <t>PHASE_2_6_A6_REPORT_CREDIBILITY_CLOSURE.md (landed on main at 66b84e4, 214 lines)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: 2.7 scaffold governance — roadmap In Progress, Sprint 0 subtasks, progress doc
Roadmap:
  - 2.7 Status: Next → In Progress
  - Sprint 0: added subtasks 2.7.a-d with SUCCESS CRITERIA, TEST METHOD, OUTPUT ARTIFACT
  - README: In Progress count 0 → 1, Next count 8 → 7, added 2.7 evidence line
  - Markdown companion regenerated

New:
  - PHASE_2_7_EVALUATION_UPLIFT_PROGRESS.md — what was built, what was proven, what remains
</commit_message>
<xml_diff>
--- a/RevisionGrade_Roadmap_UPDATED.xlsx
+++ b/RevisionGrade_Roadmap_UPDATED.xlsx
@@ -1398,7 +1398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A85"/>
+  <dimension ref="A1:A86"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="133.88" customWidth="1" style="95" min="1" max="1"/>
@@ -1446,6 +1446,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8" ht="14.25" customHeight="1" s="96">
       <c r="A8" s="95" t="inlineStr">
         <is>
@@ -1453,6 +1454,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="14.25" customHeight="1" s="96">
       <c r="A10" s="95" t="inlineStr">
         <is>
@@ -1470,14 +1472,14 @@
     <row r="12" ht="14.25" customHeight="1" s="96">
       <c r="A12" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  In Progress: 0 items</t>
+          <t xml:space="preserve">  In Progress: 1 item (2.7)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1" s="96">
       <c r="A13" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Next: 8 items</t>
+          <t xml:space="preserve">  Next: 7 items</t>
         </is>
       </c>
     </row>
@@ -1495,6 +1497,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="14.25" customHeight="1" s="96">
       <c r="A17" s="95" t="inlineStr">
         <is>
@@ -1530,6 +1533,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="14.25" customHeight="1" s="96">
       <c r="A23" s="95" t="inlineStr">
         <is>
@@ -1579,6 +1583,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31" ht="14.25" customHeight="1" s="96">
       <c r="A31" s="95" t="inlineStr">
         <is>
@@ -1643,274 +1648,281 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="95" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Canon Integration (Phase 0): NEXT</t>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Evaluation Uplift (2.7): IN PROGRESS — scaffold complete (6 suites, 52 tests, a6f0492→c91f26c, 2026-03-19)</t>
         </is>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1" s="96">
       <c r="A41" s="95" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Canon Integration (Phase 0): NEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="14.25" customHeight="1" s="96">
+      <c r="A42" s="95" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Trust &amp; Quality Uplift: NEXT IN QUEUE</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="14.25" customHeight="1" s="96"/>
-    <row r="43" ht="14.25" customHeight="1" s="96">
-      <c r="A43" s="95" t="inlineStr">
+    <row r="43" ht="14.25" customHeight="1" s="96"/>
+    <row r="44" ht="14.25" customHeight="1" s="96">
+      <c r="A44" s="95" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="14.25" customHeight="1" s="96"/>
-    <row r="45">
-      <c r="A45" s="95" t="inlineStr">
-        <is>
-          <t>Three-Layer Execution Structure</t>
-        </is>
-      </c>
-    </row>
+    <row r="45"/>
     <row r="46" ht="14.25" customHeight="1" s="96">
       <c r="A46" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Layer 1 — Roadmap: direction + sequencing (this workbook)</t>
+          <t>Three-Layer Execution Structure</t>
         </is>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1" s="96">
       <c r="A47" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Layer 2 — Sprint: atomic subtasks with verification (Sprint 0 sheet)</t>
+          <t xml:space="preserve">  Layer 1 — Roadmap: direction + sequencing (this workbook)</t>
         </is>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1" s="96">
       <c r="A48" s="95" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Layer 2 — Sprint: atomic subtasks with verification (Sprint 0 sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="14.25" customHeight="1" s="96">
+      <c r="A49" s="95" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Layer 3 — Authority: canon enforcement at runtime (Phase 0 items)</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="14.25" customHeight="1" s="96"/>
-    <row r="50" ht="14.25" customHeight="1" s="96">
-      <c r="A50" s="95" t="inlineStr">
-        <is>
-          <t>Governance Model</t>
-        </is>
-      </c>
-    </row>
+    <row r="50" ht="14.25" customHeight="1" s="96"/>
     <row r="51">
       <c r="A51" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Every roadmap item has: Success Criteria, Test Method, Canon Reference</t>
+          <t>Governance Model</t>
         </is>
       </c>
     </row>
     <row r="52" ht="14.25" customHeight="1" s="96">
       <c r="A52" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Every sprint subtask has: Success Criteria, Test Method, Output Artifact</t>
+          <t xml:space="preserve">  Every roadmap item has: Success Criteria, Test Method, Canon Reference</t>
         </is>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1" s="96">
       <c r="A53" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Definition of done: "This passed its defined success test" — not "I think this is done"</t>
+          <t xml:space="preserve">  Every sprint subtask has: Success Criteria, Test Method, Output Artifact</t>
         </is>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1" s="96">
       <c r="A54" s="95" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Definition of done: "This passed its defined success test" — not "I think this is done"</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="14.25" customHeight="1" s="96">
+      <c r="A55" s="95" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Canon compliance check required before any phase can be marked verified</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="14.25" customHeight="1" s="96"/>
-    <row r="56" ht="14.25" customHeight="1" s="96">
-      <c r="A56" s="95" t="inlineStr">
-        <is>
-          <t>Active Gates</t>
-        </is>
-      </c>
-    </row>
+    <row r="56" ht="14.25" customHeight="1" s="96"/>
     <row r="57">
       <c r="A57" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2.1 DB Verification: phase21-db-verification.sql must pass before 2.2 begins</t>
+          <t>Active Gates</t>
         </is>
       </c>
     </row>
     <row r="58" ht="14.25" customHeight="1" s="96">
       <c r="A58" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Canon Gate (Pass 1.5): Must execute before results surface to users</t>
+          <t xml:space="preserve">  2.1 DB Verification: phase21-db-verification.sql must pass before 2.2 begins</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Two-AI Independence: Pass 2 must never receive Pass 1 outputs</t>
+          <t xml:space="preserve">  Canon Gate (Pass 1.5): Must execute before results surface to users</t>
         </is>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1" s="96">
       <c r="A60" s="95" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Two-AI Independence: Pass 2 must never receive Pass 1 outputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="14.25" customHeight="1" s="96">
+      <c r="A61" s="95" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Audit Spine: Append-only, hash-chained, no DELETE/UPDATE, 7-year retention</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="14.25" customHeight="1" s="96"/>
-    <row r="62" ht="14.25" customHeight="1" s="96">
-      <c r="A62" s="95" t="inlineStr">
+    <row r="62" ht="14.25" customHeight="1" s="96"/>
+    <row r="63" ht="14.25" customHeight="1" s="96">
+      <c r="A63" s="95" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="14.25" customHeight="1" s="96"/>
-    <row r="64" ht="14.25" customHeight="1" s="96">
-      <c r="A64" s="95" t="inlineStr">
-        <is>
-          <t>Workbook Sheets</t>
-        </is>
-      </c>
-    </row>
+    <row r="64" ht="14.25" customHeight="1" s="96"/>
     <row r="65" ht="14.25" customHeight="1" s="96">
       <c r="A65" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Overview: Dashboard with KPI cards and phase progress</t>
+          <t>Workbook Sheets</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Roadmap: Full 44-item sequential tracker with all PM fields + Canon Reference</t>
+          <t xml:space="preserve">  Overview: Dashboard with KPI cards and phase progress</t>
         </is>
       </c>
     </row>
     <row r="67" ht="14.25" customHeight="1" s="96">
       <c r="A67" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Sprint 0 (Phase 2): 18 atomic subtasks for 2.1-2.6 with Success/Test/Artifact</t>
+          <t xml:space="preserve">  Roadmap: Full 44-item sequential tracker with all PM fields + Canon Reference</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Immediate Priorities: The 'next three' critical deliverables</t>
+          <t xml:space="preserve">  Sprint 0 (Phase 2): 18 atomic subtasks for 2.1-2.6 with Success/Test/Artifact</t>
         </is>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1" s="96">
       <c r="A69" s="95" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Immediate Priorities: The 'next three' critical deliverables</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="14.25" customHeight="1" s="96">
+      <c r="A70" s="95" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Canon Reference: Authority chain, numeric constants, 10 non-negotiable governance rules</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="14.25" customHeight="1" s="96"/>
-    <row r="71" ht="14.25" customHeight="1" s="96">
-      <c r="A71" s="95" t="inlineStr">
+    <row r="71" ht="14.25" customHeight="1" s="96"/>
+    <row r="72" ht="14.25" customHeight="1" s="96">
+      <c r="A72" s="95" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="14.25" customHeight="1" s="96"/>
-    <row r="73" ht="14.25" customHeight="1" s="96">
-      <c r="A73" s="95" t="inlineStr">
-        <is>
-          <t>Canon Document Sources (20 documents integrated)</t>
-        </is>
-      </c>
-    </row>
+    <row r="73" ht="14.25" customHeight="1" s="96"/>
     <row r="74" ht="14.25" customHeight="1" s="96">
       <c r="A74" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume I — WAVE Revision Guide Canon (62 waves, 3 tsunamis, 10 execution rules)</t>
+          <t>Canon Document Sources (20 documents integrated)</t>
         </is>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1" s="96">
       <c r="A75" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume II — Story Evaluation Criteria (13 criteria, 10 diagnostic patterns)</t>
+          <t xml:space="preserve">  Volume I — WAVE Revision Guide Canon (62 waves, 3 tsunamis, 10 execution rules)</t>
         </is>
       </c>
     </row>
     <row r="76" ht="14.25" customHeight="1" s="96">
       <c r="A76" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume II-A — Operational Schema (weights, gates, JSON envelope, Supabase tables)</t>
+          <t xml:space="preserve">  Volume II — Story Evaluation Criteria (13 criteria, 10 diagnostic patterns)</t>
         </is>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1" s="96">
       <c r="A77" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume III — Platform Governance Canon (5 doctrines, 3-layer editorial intelligence)</t>
+          <t xml:space="preserve">  Volume II-A — Operational Schema (weights, gates, JSON envelope, Supabase tables)</t>
         </is>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1" s="96">
       <c r="A78" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume III — Tools &amp; Implementation Systems (schemas, prompts, adapters)</t>
+          <t xml:space="preserve">  Volume III — Platform Governance Canon (5 doctrines, 3-layer editorial intelligence)</t>
         </is>
       </c>
     </row>
     <row r="79" ht="14.25" customHeight="1" s="96">
       <c r="A79" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume III — Operational Specification (thresholds, routing, 7-stage pipeline)</t>
+          <t xml:space="preserve">  Volume III — Tools &amp; Implementation Systems (schemas, prompts, adapters)</t>
         </is>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1" s="96">
       <c r="A80" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume IV — AI Governance Canon (3-layer authority, 7 protection systems)</t>
+          <t xml:space="preserve">  Volume III — Operational Specification (thresholds, routing, 7-stage pipeline)</t>
         </is>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1" s="96">
       <c r="A81" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume V — Execution Architecture (AEP 6-step flow, Trifecta, chunking, reliability)</t>
+          <t xml:space="preserve">  Volume IV — AI Governance Canon (3-layer authority, 7 protection systems)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Canon III — Lessons of the Living System (8 governing laws)</t>
+          <t xml:space="preserve">  Volume V — Execution Architecture (AEP 6-step flow, Trifecta, chunking, reliability)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Canon Assembly Matrix (RCAM v2.0, 24 source docs, 5 matrix rules)</t>
+          <t xml:space="preserve">  Canon III — Lessons of the Living System (8 governing laws)</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="95" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Canon Doctrine Registry (77 doctrine units, 6 governance rules)</t>
+          <t xml:space="preserve">  Canon Assembly Matrix (RCAM v2.0, 24 source docs, 5 matrix rules)</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Canon Doctrine Registry (77 doctrine units, 6 governance rules)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="95" t="inlineStr">
         <is>
           <t xml:space="preserve">  + 9 supporting/variant documents (txt, md formats)</t>
         </is>
@@ -3341,7 +3353,7 @@
       <c r="E13" s="137" t="n"/>
       <c r="F13" s="147" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G13" s="149" t="inlineStr">
@@ -3384,7 +3396,11 @@
           <t>Dual-axis scores. Zero generic recommendations. All recs anchored to specific text. Quality guards pass CI.</t>
         </is>
       </c>
-      <c r="O13" s="140" t="n"/>
+      <c r="O13" s="140" t="inlineStr">
+        <is>
+          <t>6 test suites: pass1, pass2, pass3, pipeline-e2e, pipeline-independence, quality-gate. 52 tests total. Pure parser tests + DI runner tests + deterministic quality gate. npm test -- tests/evaluation/pipeline/ --runInBand</t>
+        </is>
+      </c>
       <c r="P13" s="140" t="inlineStr">
         <is>
           <t>No</t>
@@ -3392,7 +3408,7 @@
       </c>
       <c r="Q13" s="140" t="inlineStr">
         <is>
-          <t>This is what makes the product feel like a senior editor, not a rubric engine.</t>
+          <t>IN PROGRESS at a6f0492, 9ef8afe, c91f26c (2026-03-19). Pipeline scaffold implemented: Pass 1, Pass 2, Pass 3, orchestration runner, prompts, quality gate, and deterministic parser-level test seams. Jest/SWC mock-hoisting issue removed via dependency injection and pure parser tests. Pipeline suite green: 6 suites, 52 tests passing.</t>
         </is>
       </c>
       <c r="R13" s="141" t="inlineStr">
@@ -5966,7 +5982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:T32"/>
+  <dimension ref="A1:T36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="95" min="1" max="1"/>
@@ -7360,6 +7376,214 @@
       <c r="H32" s="174" t="n"/>
       <c r="I32" s="174" t="n"/>
       <c r="J32" s="174" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Pipeline Scaffold</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2.7.a</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Pass 1/2/3 runners + prompt templates + types</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>lib/evaluation/pipeline/</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>runPass1, runPass2, runPass3Synthesis exported and callable with DI seam</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>pass1.test.ts, pass2.test.ts, pass3.test.ts — pure parser + DI runner tests</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>9 lib files: runPass1.ts, runPass2.ts, runPass3Synthesis.ts, runPipeline.ts, qualityGate.ts, types.ts, 3 prompt files</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Pipeline Scaffold</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2.7.b</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Quality gate (10 deterministic checks, no AI)</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>lib/evaluation/pipeline/qualityGate.ts</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>All 10 QG checks pass on valid synthesis, fail on invalid. No AI calls.</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>quality-gate.test.ts — 15 tests covering all error codes</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>qualityGate.ts (214 lines), quality-gate.test.ts (345 lines)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Pipeline Scaffold</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>2.7.c</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Pipeline orchestrator + EvaluationResultV1 adapter</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>lib/evaluation/pipeline/runPipeline.ts</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>runPipeline orchestrates Pass 1→2→3→4, returns PipelineResult union. synthesisToEvaluationResult maps to V1 schema.</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>pipeline-e2e.test.ts (7 tests), pipeline-independence.test.ts (4 tests)</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>runPipeline.ts (241 lines) with _runners DI seam</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Test Harness</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2.7.d</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Jest/SWC mock-hoisting fix — DI refactor, zero jest.mock</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>tests/evaluation/pipeline/</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>52/52 tests pass. Zero jest.mock calls. Pure parser tests + DI runner injection.</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>npm test -- tests/evaluation/pipeline/ --runInBand → 6 suites, 52 tests, all green</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>6 test files, 52 tests. Commits: a6f0492, 9ef8afe, c91f26c</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:J14"/>

</xml_diff>

<commit_message>
roadmap: update 2.7 subtasks (e-i), mark a-e complete, note blockers
Added 2.7.e (model threading — Complete), 2.7.f (real-run CLI — Complete),
2.7.g (live evidence run — Blocked on OPENAI_API_KEY), 2.7.h (independence
gate calibration — Pending), 2.7.i (final closure — Pending).

Marked existing 2.7.a-d as Complete.
Phase 2.7 status: checkpointed, not closed.
54/54 pipeline tests passing.
</commit_message>
<xml_diff>
--- a/RevisionGrade_Roadmap_UPDATED.xlsx
+++ b/RevisionGrade_Roadmap_UPDATED.xlsx
@@ -1446,7 +1446,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="14.25" customHeight="1" s="96">
       <c r="A8" s="95" t="inlineStr">
         <is>
@@ -1454,7 +1453,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="14.25" customHeight="1" s="96">
       <c r="A10" s="95" t="inlineStr">
         <is>
@@ -1497,7 +1495,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="14.25" customHeight="1" s="96">
       <c r="A17" s="95" t="inlineStr">
         <is>
@@ -1533,7 +1530,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="14.25" customHeight="1" s="96">
       <c r="A23" s="95" t="inlineStr">
         <is>
@@ -1583,7 +1579,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31" ht="14.25" customHeight="1" s="96">
       <c r="A31" s="95" t="inlineStr">
         <is>
@@ -1648,7 +1643,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="95" t="inlineStr">
         <is>
           <t xml:space="preserve">  Evaluation Uplift (2.7): IN PROGRESS — scaffold complete (6 suites, 52 tests, a6f0492→c91f26c, 2026-03-19)</t>
         </is>
@@ -1676,7 +1671,6 @@
         </is>
       </c>
     </row>
-    <row r="45"/>
     <row r="46" ht="14.25" customHeight="1" s="96">
       <c r="A46" s="95" t="inlineStr">
         <is>
@@ -5957,6 +5951,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47" ht="15" customHeight="1" s="96">
       <c r="A47" s="123" t="inlineStr">
         <is>
@@ -5982,7 +5977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:T36"/>
+  <dimension ref="A1:T41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="95" min="1" max="1"/>
@@ -6042,7 +6037,11 @@
           <t>Output Artifact</t>
         </is>
       </c>
-      <c r="K1" s="168" t="n"/>
+      <c r="K1" s="168" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
       <c r="L1" s="168" t="n"/>
       <c r="M1" s="168" t="n"/>
       <c r="N1" s="168" t="n"/>
@@ -7378,210 +7377,455 @@
       <c r="J32" s="174" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="95" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="95" t="inlineStr">
         <is>
           <t>2.7</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="95" t="inlineStr">
         <is>
           <t>Pipeline Scaffold</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="95" t="inlineStr">
         <is>
           <t>2.7.a</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="95" t="inlineStr">
         <is>
           <t>Pass 1/2/3 runners + prompt templates + types</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="95" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G33" s="95" t="inlineStr">
         <is>
           <t>lib/evaluation/pipeline/</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="H33" s="95" t="inlineStr">
         <is>
           <t>runPass1, runPass2, runPass3Synthesis exported and callable with DI seam</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="I33" s="95" t="inlineStr">
         <is>
           <t>pass1.test.ts, pass2.test.ts, pass3.test.ts — pure parser + DI runner tests</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="J33" s="95" t="inlineStr">
         <is>
           <t>9 lib files: runPass1.ts, runPass2.ts, runPass3Synthesis.ts, runPipeline.ts, qualityGate.ts, types.ts, 3 prompt files</t>
         </is>
       </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="95" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="95" t="inlineStr">
         <is>
           <t>2.7</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="95" t="inlineStr">
         <is>
           <t>Pipeline Scaffold</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="95" t="inlineStr">
         <is>
           <t>2.7.b</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="95" t="inlineStr">
         <is>
           <t>Quality gate (10 deterministic checks, no AI)</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="95" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G34" s="95" t="inlineStr">
         <is>
           <t>lib/evaluation/pipeline/qualityGate.ts</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H34" s="95" t="inlineStr">
         <is>
           <t>All 10 QG checks pass on valid synthesis, fail on invalid. No AI calls.</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="I34" s="95" t="inlineStr">
         <is>
           <t>quality-gate.test.ts — 15 tests covering all error codes</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="J34" s="95" t="inlineStr">
         <is>
           <t>qualityGate.ts (214 lines), quality-gate.test.ts (345 lines)</t>
         </is>
       </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="95" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="95" t="inlineStr">
         <is>
           <t>2.7</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="95" t="inlineStr">
         <is>
           <t>Pipeline Scaffold</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="95" t="inlineStr">
         <is>
           <t>2.7.c</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="95" t="inlineStr">
         <is>
           <t>Pipeline orchestrator + EvaluationResultV1 adapter</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" s="95" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G35" s="95" t="inlineStr">
         <is>
           <t>lib/evaluation/pipeline/runPipeline.ts</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="H35" s="95" t="inlineStr">
         <is>
           <t>runPipeline orchestrates Pass 1→2→3→4, returns PipelineResult union. synthesisToEvaluationResult maps to V1 schema.</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="I35" s="95" t="inlineStr">
         <is>
           <t>pipeline-e2e.test.ts (7 tests), pipeline-independence.test.ts (4 tests)</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="J35" s="95" t="inlineStr">
         <is>
           <t>runPipeline.ts (241 lines) with _runners DI seam</t>
         </is>
       </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="95" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="95" t="inlineStr">
         <is>
           <t>2.7</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="95" t="inlineStr">
         <is>
           <t>Test Harness</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="95" t="inlineStr">
         <is>
           <t>2.7.d</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E36" s="95" t="inlineStr">
         <is>
           <t>Jest/SWC mock-hoisting fix — DI refactor, zero jest.mock</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" s="95" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G36" s="95" t="inlineStr">
         <is>
           <t>tests/evaluation/pipeline/</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H36" s="95" t="inlineStr">
         <is>
           <t>52/52 tests pass. Zero jest.mock calls. Pure parser tests + DI runner injection.</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="I36" s="95" t="inlineStr">
         <is>
           <t>npm test -- tests/evaluation/pipeline/ --runInBand → 6 suites, 52 tests, all green</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="J36" s="95" t="inlineStr">
         <is>
           <t>6 test files, 52 tests. Commits: a6f0492, 9ef8afe, c91f26c</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>0</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Pipeline Hardening</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2.7.e</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Model override threading — end-to-end configurable model per pipeline run</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>lib/evaluation/pipeline/*.ts</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>model?: string threaded through runPass1/2/3 + runPipeline. Tested in pass1.test.ts + pipeline-e2e.test.ts</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>0</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Pipeline Hardening</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2.7.f</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Real-run CLI upgrade — artifact emission (raw, parsed, usage, quality gate)</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>scripts/pipeline/run-phase2-7-real-run.ts</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>CLI accepts --input/--title/--work-type/--model/--output-dir. Emits full artifact set.</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>0</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Evidence &amp; Closure</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2.7.g</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Fresh live evidence run — full artifact set with upgraded pipeline</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>docs/operations/evidence/runs/</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>quality_gate.json + pipeline_result.json + usage.json all present. Independence gate passes.</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Blocked (OPENAI_API_KEY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>0</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Evidence &amp; Closure</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>2.7.h</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Independence gate calibration — exclude manuscript-sourced phrases from n-gram check</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>lib/evaluation/pipeline/qualityGate.ts</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Independence check no longer flags natural language convergence. Only flags actual pass-to-pass leakage.</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>0</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Evidence &amp; Closure</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2.7.i</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Phase 2.7 final closure — flip PHASE_2_7_EVALUATION_UPLIFT_CLOSURE.md to COMPLETED</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>PHASE_2_7_EVALUATION_UPLIFT_CLOSURE.md</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Closure doc marked COMPLETED with all evidence artifacts referenced.</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
roadmap: mark 2.7.h (independence gate calibration) complete
Copilot calibrated the independence gate at b625c89:
- n-gram size increased from 6 to 8
- manuscript-sourced evidence snippets excluded from overlap check
- requires 2+ non-evidence overlaps per criterion to trigger violation
- 56/56 tests passing post-calibration

Remaining blockers: 2.7.g (live run — needs OPENAI_API_KEY), 2.7.i (closure)
</commit_message>
<xml_diff>
--- a/RevisionGrade_Roadmap_UPDATED.xlsx
+++ b/RevisionGrade_Roadmap_UPDATED.xlsx
@@ -5951,7 +5951,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47" ht="15" customHeight="1" s="96">
       <c r="A47" s="123" t="inlineStr">
         <is>
@@ -7427,7 +7426,7 @@
           <t>9 lib files: runPass1.ts, runPass2.ts, runPass3Synthesis.ts, runPipeline.ts, qualityGate.ts, types.ts, 3 prompt files</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="K33" s="95" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -7484,7 +7483,7 @@
           <t>qualityGate.ts (214 lines), quality-gate.test.ts (345 lines)</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="K34" s="95" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -7541,7 +7540,7 @@
           <t>runPipeline.ts (241 lines) with _runners DI seam</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="K35" s="95" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -7598,232 +7597,232 @@
           <t>6 test files, 52 tests. Commits: a6f0492, 9ef8afe, c91f26c</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="K36" s="95" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="n">
+      <c r="A37" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="95" t="inlineStr">
         <is>
           <t>2.7</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="95" t="inlineStr">
         <is>
           <t>Pipeline Hardening</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="95" t="inlineStr">
         <is>
           <t>2.7.e</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="95" t="inlineStr">
         <is>
           <t>Model override threading — end-to-end configurable model per pipeline run</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F37" s="95" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G37" s="95" t="inlineStr">
         <is>
           <t>lib/evaluation/pipeline/*.ts</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H37" s="95" t="inlineStr">
         <is>
           <t>model?: string threaded through runPass1/2/3 + runPipeline. Tested in pass1.test.ts + pipeline-e2e.test.ts</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="K37" s="95" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="n">
+      <c r="A38" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="95" t="inlineStr">
         <is>
           <t>2.7</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="95" t="inlineStr">
         <is>
           <t>Pipeline Hardening</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="95" t="inlineStr">
         <is>
           <t>2.7.f</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E38" s="95" t="inlineStr">
         <is>
           <t>Real-run CLI upgrade — artifact emission (raw, parsed, usage, quality gate)</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F38" s="95" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="G38" s="95" t="inlineStr">
         <is>
           <t>scripts/pipeline/run-phase2-7-real-run.ts</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="H38" s="95" t="inlineStr">
         <is>
           <t>CLI accepts --input/--title/--work-type/--model/--output-dir. Emits full artifact set.</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="K38" s="95" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="n">
+      <c r="A39" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="95" t="inlineStr">
         <is>
           <t>2.7</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="95" t="inlineStr">
         <is>
           <t>Evidence &amp; Closure</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="95" t="inlineStr">
         <is>
           <t>2.7.g</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" s="95" t="inlineStr">
         <is>
           <t>Fresh live evidence run — full artifact set with upgraded pipeline</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" s="95" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G39" s="95" t="inlineStr">
         <is>
           <t>docs/operations/evidence/runs/</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H39" s="95" t="inlineStr">
         <is>
           <t>quality_gate.json + pipeline_result.json + usage.json all present. Independence gate passes.</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="K39" s="95" t="inlineStr">
         <is>
           <t>Blocked (OPENAI_API_KEY)</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="n">
+      <c r="A40" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="95" t="inlineStr">
         <is>
           <t>2.7</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="95" t="inlineStr">
         <is>
           <t>Evidence &amp; Closure</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="95" t="inlineStr">
         <is>
           <t>2.7.h</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E40" s="95" t="inlineStr">
         <is>
           <t>Independence gate calibration — exclude manuscript-sourced phrases from n-gram check</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F40" s="95" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G40" s="95" t="inlineStr">
         <is>
           <t>lib/evaluation/pipeline/qualityGate.ts</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="H40" s="95" t="inlineStr">
         <is>
           <t>Independence check no longer flags natural language convergence. Only flags actual pass-to-pass leakage.</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="K40" s="95" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="n">
+      <c r="A41" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="95" t="inlineStr">
         <is>
           <t>2.7</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="95" t="inlineStr">
         <is>
           <t>Evidence &amp; Closure</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="95" t="inlineStr">
         <is>
           <t>2.7.i</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E41" s="95" t="inlineStr">
         <is>
           <t>Phase 2.7 final closure — flip PHASE_2_7_EVALUATION_UPLIFT_CLOSURE.md to COMPLETED</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="95" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G41" s="95" t="inlineStr">
         <is>
           <t>PHASE_2_7_EVALUATION_UPLIFT_CLOSURE.md</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H41" s="95" t="inlineStr">
         <is>
           <t>Closure doc marked COMPLETED with all evidence artifacts referenced.</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="K41" s="95" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>

</xml_diff>

<commit_message>
phase 2.7: CLOSED — evaluation uplift complete
Phase 2.7 closure doc flipped to COMPLETED.
All 9 subtasks (2.7.a through 2.7.i) marked Complete.
Roadmap updated: Phase 2.7 → Complete.

Deliverables: 4-pass dual-axis pipeline, 10-check quality gate,
calibrated independence guarantee, EvaluationResultV1 backward
compatibility, model override threading, real-run CLI, archived
evidence pack, 56/56 tests passing.

Three-tool collaboration: Copilot (implementation), ChatGPT (spec +
prompt design + calibration recommendation), Perplexity (verification +
governance + roadmap).
</commit_message>
<xml_diff>
--- a/RevisionGrade_Roadmap_UPDATED.xlsx
+++ b/RevisionGrade_Roadmap_UPDATED.xlsx
@@ -5951,6 +5951,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47" ht="15" customHeight="1" s="96">
       <c r="A47" s="123" t="inlineStr">
         <is>
@@ -7734,7 +7735,7 @@
       </c>
       <c r="K39" s="95" t="inlineStr">
         <is>
-          <t>Blocked (OPENAI_API_KEY)</t>
+          <t>Complete</t>
         </is>
       </c>
     </row>
@@ -7824,7 +7825,7 @@
       </c>
       <c r="K41" s="95" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
roadmap: Phase 0.1 (Canon Registry Binding) — COMPLETE
PR #39 merged at 57a6d97. Added 7 subtasks (0.1.a-g), all Complete.
58/58 tests passing. Registry is runtime-bound, fail-closed,
injected into all passes, with timeout enforcement.

Next: Phase 0.2 (Lessons Learned Rule Engine) or Phase 2.8 (Multi-Chunk).
</commit_message>
<xml_diff>
--- a/RevisionGrade_Roadmap_UPDATED.xlsx
+++ b/RevisionGrade_Roadmap_UPDATED.xlsx
@@ -5977,7 +5977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:T41"/>
+  <dimension ref="A1:T48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="95" min="1" max="1"/>
@@ -7824,6 +7824,293 @@
         </is>
       </c>
       <c r="K41" s="95" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>0</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Canon Registry Binding</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>0.1.a</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Canon registry types + static entries (16 entries)</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>lib/governance/canonRegistry.ts</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>0</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Canon Registry Binding</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>0.1.b</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>validateCanonicalRegistry() — fail-closed structural validation</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>lib/governance/canonRegistry.ts</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>0</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Canon Registry Binding</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>0.1.c</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>loadCanonicalRegistry() + readonly facade + freeze-on-boot</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>lib/governance/canonRegistry.ts</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>0</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Canon Registry Binding</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>0.1.d</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Pipeline registry binding — load before passes, fail-closed</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>lib/evaluation/pipeline/runPipeline.ts</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>0</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Canon Registry Binding</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>0.1.e</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Registry injection into Pass 1/2/3 — required, not optional</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>lib/evaluation/pipeline/runPass1-3.ts</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>0</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Canon Registry Binding</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>0.1.f</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Input validation + per-pass timeout enforcement</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>lib/evaluation/pipeline/runPipeline.ts</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>0</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Canon Registry Binding</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>0.1.g</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Tests: fail-closed binding, invalid input, timeout, registry immutability</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>tests/evaluation/pipeline/</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>

</xml_diff>

<commit_message>
roadmap: Phase 0.2 (Lessons Learned Rule Engine) — COMPLETE
PR #40 merged at 162b188. Added 9 subtasks (0.2.a-i), all Complete.
5 mandatory rules, 4 pipeline injection points, fail-closed enforcement.
21/21 focused tests passing. Closure report included.

Next: Phase 0.3 (Governance Injection Map) or Phase 2.8 (Multi-Chunk).
Note: 3 pre-existing legacy test failures need separate fix.
</commit_message>
<xml_diff>
--- a/RevisionGrade_Roadmap_UPDATED.xlsx
+++ b/RevisionGrade_Roadmap_UPDATED.xlsx
@@ -5977,7 +5977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:T48"/>
+  <dimension ref="A1:T57"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="95" min="1" max="1"/>
@@ -7830,287 +7830,647 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="n">
+      <c r="A42" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="95" t="inlineStr">
         <is>
           <t>0.1</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="95" t="inlineStr">
         <is>
           <t>Canon Registry Binding</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="95" t="inlineStr">
         <is>
           <t>0.1.a</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E42" s="95" t="inlineStr">
         <is>
           <t>Canon registry types + static entries (16 entries)</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" s="95" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G42" s="95" t="inlineStr">
         <is>
           <t>lib/governance/canonRegistry.ts</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="K42" t="inlineStr">
+      <c r="H42" s="95" t="inlineStr"/>
+      <c r="K42" s="95" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="n">
+      <c r="A43" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="95" t="inlineStr">
         <is>
           <t>0.1</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="95" t="inlineStr">
         <is>
           <t>Canon Registry Binding</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="95" t="inlineStr">
         <is>
           <t>0.1.b</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E43" s="95" t="inlineStr">
         <is>
           <t>validateCanonicalRegistry() — fail-closed structural validation</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" s="95" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="G43" s="95" t="inlineStr">
         <is>
           <t>lib/governance/canonRegistry.ts</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="K43" t="inlineStr">
+      <c r="H43" s="95" t="inlineStr"/>
+      <c r="K43" s="95" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="n">
+      <c r="A44" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="95" t="inlineStr">
         <is>
           <t>0.1</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="95" t="inlineStr">
         <is>
           <t>Canon Registry Binding</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="95" t="inlineStr">
         <is>
           <t>0.1.c</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E44" s="95" t="inlineStr">
         <is>
           <t>loadCanonicalRegistry() + readonly facade + freeze-on-boot</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F44" s="95" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G44" s="95" t="inlineStr">
         <is>
           <t>lib/governance/canonRegistry.ts</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="K44" t="inlineStr">
+      <c r="H44" s="95" t="inlineStr"/>
+      <c r="K44" s="95" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="n">
+      <c r="A45" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="95" t="inlineStr">
         <is>
           <t>0.1</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="95" t="inlineStr">
         <is>
           <t>Canon Registry Binding</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="95" t="inlineStr">
         <is>
           <t>0.1.d</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E45" s="95" t="inlineStr">
         <is>
           <t>Pipeline registry binding — load before passes, fail-closed</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="95" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G45" s="95" t="inlineStr">
         <is>
           <t>lib/evaluation/pipeline/runPipeline.ts</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="K45" t="inlineStr">
+      <c r="H45" s="95" t="inlineStr"/>
+      <c r="K45" s="95" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="n">
+      <c r="A46" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="95" t="inlineStr">
         <is>
           <t>0.1</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="95" t="inlineStr">
         <is>
           <t>Canon Registry Binding</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="95" t="inlineStr">
         <is>
           <t>0.1.e</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E46" s="95" t="inlineStr">
         <is>
           <t>Registry injection into Pass 1/2/3 — required, not optional</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F46" s="95" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="G46" s="95" t="inlineStr">
         <is>
           <t>lib/evaluation/pipeline/runPass1-3.ts</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
-      <c r="K46" t="inlineStr">
+      <c r="H46" s="95" t="inlineStr"/>
+      <c r="K46" s="95" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="n">
+      <c r="A47" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="95" t="inlineStr">
         <is>
           <t>0.1</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="95" t="inlineStr">
         <is>
           <t>Canon Registry Binding</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="95" t="inlineStr">
         <is>
           <t>0.1.f</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E47" s="95" t="inlineStr">
         <is>
           <t>Input validation + per-pass timeout enforcement</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" s="95" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="G47" s="95" t="inlineStr">
         <is>
           <t>lib/evaluation/pipeline/runPipeline.ts</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="K47" t="inlineStr">
+      <c r="H47" s="95" t="inlineStr"/>
+      <c r="K47" s="95" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="n">
+      <c r="A48" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="95" t="inlineStr">
         <is>
           <t>0.1</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="95" t="inlineStr">
         <is>
           <t>Canon Registry Binding</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="95" t="inlineStr">
         <is>
           <t>0.1.g</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E48" s="95" t="inlineStr">
         <is>
           <t>Tests: fail-closed binding, invalid input, timeout, registry immutability</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F48" s="95" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
+      <c r="G48" s="95" t="inlineStr">
         <is>
           <t>tests/evaluation/pipeline/</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
-      <c r="K48" t="inlineStr">
+      <c r="H48" s="95" t="inlineStr"/>
+      <c r="K48" s="95" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>0</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Lessons Learned Rule Engine</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>0.2.a</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Rule contract types (LessonsLearnedRule, RuleResult, Report)</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>lib/governance/lessonsLearned/types.ts</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>0</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Lessons Learned Rule Engine</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>0.2.b</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>5 mandatory rules with predicate implementations (LLR-001 through LLR-005)</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>lib/governance/lessonsLearned/ACTIVE_RULES.ts</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>0</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Lessons Learned Rule Engine</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>0.2.c</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Rule engine — evaluateLessonsLearnedRules() + deriveDecision()</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>lib/governance/lessonsLearned/engine.ts</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>0</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Lessons Learned Rule Engine</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>0.2.d</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Pipeline injection — 4 enforcement points (post-structural, post-diagnostic, post-convergence, pre-artifact)</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>lib/evaluation/pipeline/runPipeline.ts</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>0</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Lessons Learned Rule Engine</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>0.2.e</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Fail-closed block codes (LLR_POST_STRUCTURAL_BLOCK, etc.)</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>lib/evaluation/pipeline/runPipeline.ts</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>0</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Lessons Learned Rule Engine</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>0.2.f</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Engine tests — 8 tests (5 rule failures, registration, block-on-error, pass)</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>lib/governance/__tests__/lessonsLearnedEngine.test.ts</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>0</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Lessons Learned Rule Engine</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>0.2.g</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Pipeline integration tests — stage-block behavior</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>tests/evaluation/pipeline/pipeline-e2e.test.ts</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>0</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Lessons Learned Rule Engine</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>0.2.h</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>DOMINATUS failure case calibration artifact</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Calibration</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>calibration/phase0.2/</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>0</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Lessons Learned Rule Engine</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>0.2.i</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Phase 0.2 closure report</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>PHASE_0_2_CLOSURE_REPORT.md</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>

</xml_diff>

<commit_message>
roadmap: Phase 0.3 (Governance Injection Map) — COMPLETE
PR #42 merged at 3804b24. Added 6 subtasks (0.3.a-f), all Complete.
11 required checkpoints, fail-closed validation, pipeline-bound.
13/13 suites, 156/156 tests passing.

Phase 0 enforcement stack (0.1 + 0.2 + 0.3) is now fully operational.
Next: gold-standard normalization, acceptance hardening, prompt rewrites, then 2.8.
</commit_message>
<xml_diff>
--- a/RevisionGrade_Roadmap_UPDATED.xlsx
+++ b/RevisionGrade_Roadmap_UPDATED.xlsx
@@ -5977,7 +5977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:T57"/>
+  <dimension ref="A1:T63"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="95" min="1" max="1"/>
@@ -8117,360 +8117,600 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="n">
+      <c r="A49" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="95" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="95" t="inlineStr">
         <is>
           <t>Lessons Learned Rule Engine</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="95" t="inlineStr">
         <is>
           <t>0.2.a</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E49" s="95" t="inlineStr">
         <is>
           <t>Rule contract types (LessonsLearnedRule, RuleResult, Report)</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F49" s="95" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
+      <c r="G49" s="95" t="inlineStr">
         <is>
           <t>lib/governance/lessonsLearned/types.ts</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
+      <c r="K49" s="95" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="n">
+      <c r="A50" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="95" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="95" t="inlineStr">
         <is>
           <t>Lessons Learned Rule Engine</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="95" t="inlineStr">
         <is>
           <t>0.2.b</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E50" s="95" t="inlineStr">
         <is>
           <t>5 mandatory rules with predicate implementations (LLR-001 through LLR-005)</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F50" s="95" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
+      <c r="G50" s="95" t="inlineStr">
         <is>
           <t>lib/governance/lessonsLearned/ACTIVE_RULES.ts</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
+      <c r="K50" s="95" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="n">
+      <c r="A51" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="95" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="95" t="inlineStr">
         <is>
           <t>Lessons Learned Rule Engine</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="95" t="inlineStr">
         <is>
           <t>0.2.c</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E51" s="95" t="inlineStr">
         <is>
           <t>Rule engine — evaluateLessonsLearnedRules() + deriveDecision()</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F51" s="95" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
+      <c r="G51" s="95" t="inlineStr">
         <is>
           <t>lib/governance/lessonsLearned/engine.ts</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr">
+      <c r="K51" s="95" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="n">
+      <c r="A52" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="95" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="95" t="inlineStr">
         <is>
           <t>Lessons Learned Rule Engine</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D52" s="95" t="inlineStr">
         <is>
           <t>0.2.d</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E52" s="95" t="inlineStr">
         <is>
           <t>Pipeline injection — 4 enforcement points (post-structural, post-diagnostic, post-convergence, pre-artifact)</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="F52" s="95" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
+      <c r="G52" s="95" t="inlineStr">
         <is>
           <t>lib/evaluation/pipeline/runPipeline.ts</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
+      <c r="K52" s="95" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="n">
+      <c r="A53" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="95" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="95" t="inlineStr">
         <is>
           <t>Lessons Learned Rule Engine</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D53" s="95" t="inlineStr">
         <is>
           <t>0.2.e</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E53" s="95" t="inlineStr">
         <is>
           <t>Fail-closed block codes (LLR_POST_STRUCTURAL_BLOCK, etc.)</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F53" s="95" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="G53" s="95" t="inlineStr">
         <is>
           <t>lib/evaluation/pipeline/runPipeline.ts</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr">
+      <c r="K53" s="95" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="n">
+      <c r="A54" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="95" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="95" t="inlineStr">
         <is>
           <t>Lessons Learned Rule Engine</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D54" s="95" t="inlineStr">
         <is>
           <t>0.2.f</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E54" s="95" t="inlineStr">
         <is>
           <t>Engine tests — 8 tests (5 rule failures, registration, block-on-error, pass)</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F54" s="95" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
+      <c r="G54" s="95" t="inlineStr">
         <is>
           <t>lib/governance/__tests__/lessonsLearnedEngine.test.ts</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
+      <c r="K54" s="95" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="n">
+      <c r="A55" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="95" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="95" t="inlineStr">
         <is>
           <t>Lessons Learned Rule Engine</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D55" s="95" t="inlineStr">
         <is>
           <t>0.2.g</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
+      <c r="E55" s="95" t="inlineStr">
         <is>
           <t>Pipeline integration tests — stage-block behavior</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="F55" s="95" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr">
+      <c r="G55" s="95" t="inlineStr">
         <is>
           <t>tests/evaluation/pipeline/pipeline-e2e.test.ts</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr">
+      <c r="K55" s="95" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="n">
+      <c r="A56" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B56" s="95" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C56" s="95" t="inlineStr">
         <is>
           <t>Lessons Learned Rule Engine</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D56" s="95" t="inlineStr">
         <is>
           <t>0.2.h</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="E56" s="95" t="inlineStr">
         <is>
           <t>DOMINATUS failure case calibration artifact</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="F56" s="95" t="inlineStr">
         <is>
           <t>Calibration</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr">
+      <c r="G56" s="95" t="inlineStr">
         <is>
           <t>calibration/phase0.2/</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr">
+      <c r="K56" s="95" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="n">
+      <c r="A57" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B57" s="95" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="95" t="inlineStr">
         <is>
           <t>Lessons Learned Rule Engine</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D57" s="95" t="inlineStr">
         <is>
           <t>0.2.i</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E57" s="95" t="inlineStr">
         <is>
           <t>Phase 0.2 closure report</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="F57" s="95" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr">
+      <c r="G57" s="95" t="inlineStr">
         <is>
           <t>PHASE_0_2_CLOSURE_REPORT.md</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr">
+      <c r="K57" s="95" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>0</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Governance Injection Map</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>0.3.a</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Injection map types + 11 required checkpoint definitions</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>lib/governance/injectionMap.ts</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>0</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Governance Injection Map</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>0.3.b</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Fail-closed map validation (empty, duplicates, missing required, BLOCK without error code)</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>lib/governance/injectionMap.ts</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>0</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Governance Injection Map</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>0.3.c</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Pipeline boot integration — load + validate map before passes</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>lib/evaluation/pipeline/runPipeline.ts</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>0</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Governance Injection Map</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>0.3.d</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Checkpoint context in all error paths (canon, LLR, quality gate)</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>lib/evaluation/pipeline/runPipeline.ts</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>0</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Governance Injection Map</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>0.3.e</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Injection map unit tests + pipeline integration tests</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>lib/governance/__tests__/injectionMap.test.ts</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>0</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Governance Injection Map</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>0.3.f</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Phase 0.3 governance mapping artifact</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>PHASE_0_3_GOVERNANCE_INJECTION_MAP.md</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>

</xml_diff>